<commit_message>
MAJ Plan de charge + Patrimoine
</commit_message>
<xml_diff>
--- a/Plan de charge + Patrimoine.xlsx
+++ b/Plan de charge + Patrimoine.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://15041946-my.sharepoint.com/personal/guillaume_guilbert_ext_plasticomnium_com/Documents/Documents/000-Perso/Conseil patrimoine/Outils/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{94FEFB5F-3ED6-6A40-A1A9-E7F78A9C40C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C778769B-56F8-4899-A0F1-05F0585E8A18}"/>
+  <xr:revisionPtr revIDLastSave="125" documentId="13_ncr:1_{94FEFB5F-3ED6-6A40-A1A9-E7F78A9C40C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0D604C0-BFD1-4AB4-B6F4-E558C71C5A35}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -258,7 +258,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="203">
   <si>
     <t>PLAN DE CHARGE / FLUX MENSUEL</t>
   </si>
@@ -293,9 +293,6 @@
     <t>Loyer</t>
   </si>
   <si>
-    <t xml:space="preserve">Compte Courant n°1 : </t>
-  </si>
-  <si>
     <t>Lieu de naissance :</t>
   </si>
   <si>
@@ -381,9 +378,6 @@
   </si>
   <si>
     <t>Electricité</t>
-  </si>
-  <si>
-    <t>PEE/PEG</t>
   </si>
   <si>
     <t>Internet</t>
@@ -830,9 +824,6 @@
     <t>Crédit (RP/Conso/…)</t>
   </si>
   <si>
-    <t>Nom/Prénom/Date de naissance:</t>
-  </si>
-  <si>
     <t>Capital Restant Dû</t>
   </si>
   <si>
@@ -861,6 +852,57 @@
   </si>
   <si>
     <t xml:space="preserve">Prime de départ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compte Courant n°1 [0%] : </t>
+  </si>
+  <si>
+    <t>CEL [1% brut soit 0,7% net d'IR]</t>
+  </si>
+  <si>
+    <t>PEL [2,5% net d'IR] max 10 000€</t>
+  </si>
+  <si>
+    <t>LDD [1,7% net d'IR] max 12 800€</t>
+  </si>
+  <si>
+    <t>Livret A [1,7% net d'IR] max 22 950€</t>
+  </si>
+  <si>
+    <t>Compte à terme</t>
+  </si>
+  <si>
+    <t>Epargne court terme</t>
+  </si>
+  <si>
+    <t>PEE/PEG/PEI</t>
+  </si>
+  <si>
+    <t>Epargne moyen terme</t>
+  </si>
+  <si>
+    <t>Epargne long terme</t>
+  </si>
+  <si>
+    <t>Global</t>
+  </si>
+  <si>
+    <t>Autre épargne</t>
+  </si>
+  <si>
+    <t>Budget Projets disponible</t>
+  </si>
+  <si>
+    <t>Budget Projets désiré</t>
+  </si>
+  <si>
+    <t>Prénom</t>
+  </si>
+  <si>
+    <t>Date de naissance</t>
+  </si>
+  <si>
+    <t>Non</t>
   </si>
 </sst>
 </file>
@@ -874,7 +916,7 @@
     <numFmt numFmtId="167" formatCode="#,##0&quot; €/mois&quot;"/>
     <numFmt numFmtId="168" formatCode="_ * #,##0_)\ &quot;€&quot;_ ;_ * \(#,##0\)\ &quot;€&quot;_ ;_ * &quot;-&quot;??_)\ &quot;€&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -999,24 +1041,11 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1052,8 +1081,15 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="29">
+  <fills count="30">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1220,6 +1256,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1822,7 +1864,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="198">
+  <cellXfs count="201">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1949,7 +1991,7 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="18" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2007,9 +2049,6 @@
     <xf numFmtId="0" fontId="5" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="165" fontId="1" fillId="24" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2020,42 +2059,38 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="1" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2098,8 +2133,8 @@
     <xf numFmtId="49" fontId="1" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2131,31 +2166,27 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2165,11 +2196,15 @@
     <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2180,6 +2215,22 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="29" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="29" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4472,7 +4523,7 @@
   <sheetPr>
     <tabColor rgb="FFFFD965"/>
   </sheetPr>
-  <dimension ref="A1:Z1004"/>
+  <dimension ref="A1:AA1009"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.77734375" customWidth="1"/>
@@ -4490,40 +4541,41 @@
     <col min="13" max="13" width="9.21875" customWidth="1"/>
     <col min="14" max="14" width="31.21875" customWidth="1"/>
     <col min="15" max="15" width="11.44140625" customWidth="1"/>
-    <col min="16" max="16" width="10.6640625" customWidth="1"/>
-    <col min="17" max="26" width="9.21875" customWidth="1"/>
+    <col min="16" max="17" width="10.6640625" customWidth="1"/>
+    <col min="18" max="27" width="9.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C1" s="1"/>
       <c r="D1" s="2"/>
       <c r="G1" s="3"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="142" t="s">
-        <v>186</v>
-      </c>
-      <c r="C2" s="141"/>
+    <row r="2" spans="2:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="140" t="s">
+        <v>183</v>
+      </c>
+      <c r="C2" s="139"/>
       <c r="E2" s="92"/>
-      <c r="F2" s="170" t="s">
-        <v>0</v>
-      </c>
-      <c r="G2" s="171"/>
-      <c r="H2" s="171"/>
-      <c r="I2" s="171"/>
-      <c r="J2" s="171"/>
+      <c r="F2" s="167" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="168"/>
+      <c r="H2" s="168"/>
+      <c r="I2" s="168"/>
+      <c r="J2" s="168"/>
       <c r="K2" s="92"/>
       <c r="M2" s="100"/>
-      <c r="N2" s="164" t="s">
+      <c r="N2" s="161" t="s">
         <v>1</v>
       </c>
-      <c r="O2" s="164"/>
-      <c r="P2" s="164"/>
-      <c r="Q2" s="120"/>
-    </row>
-    <row r="3" spans="2:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="132" t="s">
+      <c r="O2" s="161"/>
+      <c r="P2" s="161"/>
+      <c r="Q2" s="160"/>
+      <c r="R2" s="120"/>
+    </row>
+    <row r="3" spans="2:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="131" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="99"/>
@@ -4538,41 +4590,47 @@
       <c r="N3" s="100"/>
       <c r="O3" s="100"/>
       <c r="P3" s="100"/>
-      <c r="Q3" s="120"/>
-    </row>
-    <row r="4" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B4" s="132" t="s">
+      <c r="Q3" s="100"/>
+      <c r="R3" s="120"/>
+    </row>
+    <row r="4" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B4" s="131" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="99"/>
       <c r="E4" s="92"/>
-      <c r="F4" s="172" t="s">
+      <c r="F4" s="169" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="173"/>
+      <c r="G4" s="170"/>
       <c r="H4" s="102" t="s">
-        <v>169</v>
-      </c>
-      <c r="I4" s="174" t="s">
+        <v>167</v>
+      </c>
+      <c r="I4" s="171" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="175"/>
+      <c r="J4" s="172"/>
       <c r="K4" s="95"/>
       <c r="M4" s="100"/>
       <c r="N4" s="121" t="s">
         <v>6</v>
       </c>
-      <c r="O4" s="163" t="s">
+      <c r="O4" s="121" t="s">
         <v>7</v>
       </c>
-      <c r="P4" s="163"/>
-      <c r="Q4" s="120"/>
-    </row>
-    <row r="5" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B5" s="132" t="s">
+      <c r="P4" s="121" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q4" s="121" t="s">
+        <v>196</v>
+      </c>
+      <c r="R4" s="120"/>
+    </row>
+    <row r="5" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B5" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="133"/>
+      <c r="C5" s="132"/>
       <c r="E5" s="92"/>
       <c r="F5" s="103" t="s">
         <v>9</v>
@@ -4592,31 +4650,37 @@
       <c r="K5" s="118"/>
       <c r="M5" s="100"/>
       <c r="N5" s="53" t="s">
+        <v>186</v>
+      </c>
+      <c r="O5" s="101">
+        <v>0</v>
+      </c>
+      <c r="P5" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="101">
+        <f>SUM(O5:P5)</f>
+        <v>0</v>
+      </c>
+      <c r="R5" s="120"/>
+    </row>
+    <row r="6" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B6" s="131" t="s">
         <v>11</v>
-      </c>
-      <c r="O5" s="101">
-        <v>0</v>
-      </c>
-      <c r="P5" s="122"/>
-      <c r="Q5" s="120"/>
-    </row>
-    <row r="6" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B6" s="132" t="s">
-        <v>12</v>
       </c>
       <c r="C6" s="99"/>
       <c r="E6" s="92"/>
       <c r="F6" s="103" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="104">
+        <v>0</v>
+      </c>
+      <c r="H6" s="104">
+        <v>0</v>
+      </c>
+      <c r="I6" s="103" t="s">
         <v>13</v>
-      </c>
-      <c r="G6" s="104">
-        <v>0</v>
-      </c>
-      <c r="H6" s="104">
-        <v>0</v>
-      </c>
-      <c r="I6" s="103" t="s">
-        <v>14</v>
       </c>
       <c r="J6" s="104">
         <v>0</v>
@@ -4624,31 +4688,37 @@
       <c r="K6" s="109"/>
       <c r="M6" s="100"/>
       <c r="N6" s="53" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O6" s="101">
         <v>0</v>
       </c>
-      <c r="P6" s="122"/>
-      <c r="Q6" s="120"/>
-    </row>
-    <row r="7" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B7" s="134" t="s">
-        <v>167</v>
-      </c>
-      <c r="C7" s="162"/>
+      <c r="P6" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="101">
+        <f t="shared" ref="Q6:Q25" si="0">SUM(O6:P6)</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="120"/>
+    </row>
+    <row r="7" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B7" s="133" t="s">
+        <v>165</v>
+      </c>
+      <c r="C7" s="159"/>
       <c r="E7" s="92"/>
       <c r="F7" s="103" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="104">
+        <v>0</v>
+      </c>
+      <c r="H7" s="104">
+        <v>0</v>
+      </c>
+      <c r="I7" s="103" t="s">
         <v>16</v>
-      </c>
-      <c r="G7" s="104">
-        <v>0</v>
-      </c>
-      <c r="H7" s="104">
-        <v>0</v>
-      </c>
-      <c r="I7" s="103" t="s">
-        <v>17</v>
       </c>
       <c r="J7" s="104">
         <v>0</v>
@@ -4656,31 +4726,37 @@
       <c r="K7" s="109"/>
       <c r="M7" s="100"/>
       <c r="N7" s="53" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O7" s="101">
         <v>0</v>
       </c>
-      <c r="P7" s="122"/>
-      <c r="Q7" s="120"/>
-    </row>
-    <row r="8" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B8" s="135" t="s">
-        <v>168</v>
+      <c r="P7" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R7" s="120"/>
+    </row>
+    <row r="8" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B8" s="134" t="s">
+        <v>166</v>
       </c>
       <c r="C8" s="93"/>
       <c r="E8" s="92"/>
       <c r="F8" s="103" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="104">
+        <v>0</v>
+      </c>
+      <c r="H8" s="104">
+        <v>0</v>
+      </c>
+      <c r="I8" s="103" t="s">
         <v>20</v>
-      </c>
-      <c r="G8" s="104">
-        <v>0</v>
-      </c>
-      <c r="H8" s="104">
-        <v>0</v>
-      </c>
-      <c r="I8" s="103" t="s">
-        <v>21</v>
       </c>
       <c r="J8" s="104">
         <v>0</v>
@@ -4688,31 +4764,37 @@
       <c r="K8" s="109"/>
       <c r="M8" s="100"/>
       <c r="N8" s="53" t="s">
-        <v>22</v>
+        <v>190</v>
       </c>
       <c r="O8" s="101">
         <v>0</v>
       </c>
-      <c r="P8" s="122"/>
-      <c r="Q8" s="120"/>
-    </row>
-    <row r="9" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B9" s="135" t="s">
-        <v>162</v>
-      </c>
-      <c r="C9" s="136"/>
+      <c r="P8" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R8" s="120"/>
+    </row>
+    <row r="9" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B9" s="134" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" s="135"/>
       <c r="E9" s="92"/>
       <c r="F9" s="103" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="104">
+        <v>0</v>
+      </c>
+      <c r="H9" s="104">
+        <v>0</v>
+      </c>
+      <c r="I9" s="103" t="s">
         <v>24</v>
-      </c>
-      <c r="G9" s="104">
-        <v>0</v>
-      </c>
-      <c r="H9" s="104">
-        <v>0</v>
-      </c>
-      <c r="I9" s="103" t="s">
-        <v>25</v>
       </c>
       <c r="J9" s="104">
         <v>0</v>
@@ -4720,31 +4802,37 @@
       <c r="K9" s="109"/>
       <c r="M9" s="100"/>
       <c r="N9" s="53" t="s">
-        <v>26</v>
+        <v>189</v>
       </c>
       <c r="O9" s="101">
         <v>0</v>
       </c>
-      <c r="P9" s="122"/>
-      <c r="Q9" s="120"/>
-    </row>
-    <row r="10" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B10" s="137" t="s">
-        <v>163</v>
-      </c>
-      <c r="C10" s="138"/>
+      <c r="P9" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R9" s="120"/>
+    </row>
+    <row r="10" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B10" s="136" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="137"/>
       <c r="E10" s="92"/>
       <c r="F10" s="103" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="104">
+        <v>0</v>
+      </c>
+      <c r="H10" s="104">
+        <v>0</v>
+      </c>
+      <c r="I10" s="103" t="s">
         <v>27</v>
-      </c>
-      <c r="G10" s="104">
-        <v>0</v>
-      </c>
-      <c r="H10" s="104">
-        <v>0</v>
-      </c>
-      <c r="I10" s="103" t="s">
-        <v>28</v>
       </c>
       <c r="J10" s="104">
         <v>0</v>
@@ -4752,31 +4840,37 @@
       <c r="K10" s="109"/>
       <c r="M10" s="100"/>
       <c r="N10" s="53" t="s">
-        <v>29</v>
+        <v>187</v>
       </c>
       <c r="O10" s="101">
         <v>0</v>
       </c>
-      <c r="P10" s="122"/>
-      <c r="Q10" s="120"/>
-    </row>
-    <row r="11" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B11" s="135" t="s">
-        <v>164</v>
-      </c>
-      <c r="C11" s="136"/>
+      <c r="P10" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R10" s="120"/>
+    </row>
+    <row r="11" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B11" s="134" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" s="135"/>
       <c r="E11" s="92"/>
       <c r="F11" s="103" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="104">
+        <v>0</v>
+      </c>
+      <c r="H11" s="104">
+        <v>0</v>
+      </c>
+      <c r="I11" s="103" t="s">
         <v>30</v>
-      </c>
-      <c r="G11" s="104">
-        <v>0</v>
-      </c>
-      <c r="H11" s="104">
-        <v>0</v>
-      </c>
-      <c r="I11" s="103" t="s">
-        <v>31</v>
       </c>
       <c r="J11" s="104">
         <v>0</v>
@@ -4784,29 +4878,35 @@
       <c r="K11" s="109"/>
       <c r="M11" s="100"/>
       <c r="N11" s="53" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O11" s="101">
         <v>0</v>
       </c>
-      <c r="P11" s="122"/>
-      <c r="Q11" s="120"/>
-    </row>
-    <row r="12" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="P11" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R11" s="120"/>
+    </row>
+    <row r="12" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B12" s="93"/>
       <c r="C12" s="93"/>
       <c r="E12" s="92"/>
       <c r="F12" s="103" t="s">
+        <v>32</v>
+      </c>
+      <c r="G12" s="104">
+        <v>0</v>
+      </c>
+      <c r="H12" s="104">
+        <v>0</v>
+      </c>
+      <c r="I12" s="103" t="s">
         <v>33</v>
-      </c>
-      <c r="G12" s="104">
-        <v>0</v>
-      </c>
-      <c r="H12" s="104">
-        <v>0</v>
-      </c>
-      <c r="I12" s="103" t="s">
-        <v>34</v>
       </c>
       <c r="J12" s="104">
         <v>0</v>
@@ -4814,31 +4914,37 @@
       <c r="K12" s="109"/>
       <c r="M12" s="100"/>
       <c r="N12" s="53" t="s">
-        <v>35</v>
+        <v>188</v>
       </c>
       <c r="O12" s="101">
         <v>0</v>
       </c>
-      <c r="P12" s="122"/>
-      <c r="Q12" s="120"/>
-    </row>
-    <row r="13" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B13" s="145" t="s">
-        <v>187</v>
+      <c r="P12" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R12" s="120"/>
+    </row>
+    <row r="13" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B13" s="142" t="s">
+        <v>184</v>
       </c>
       <c r="C13" s="99"/>
       <c r="E13" s="92"/>
       <c r="F13" s="103" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="104">
+        <v>0</v>
+      </c>
+      <c r="H13" s="104">
+        <v>0</v>
+      </c>
+      <c r="I13" s="103" t="s">
         <v>36</v>
-      </c>
-      <c r="G13" s="104">
-        <v>0</v>
-      </c>
-      <c r="H13" s="104">
-        <v>0</v>
-      </c>
-      <c r="I13" s="103" t="s">
-        <v>37</v>
       </c>
       <c r="J13" s="104">
         <v>0</v>
@@ -4846,22 +4952,28 @@
       <c r="K13" s="109"/>
       <c r="M13" s="100"/>
       <c r="N13" s="53" t="s">
-        <v>38</v>
+        <v>191</v>
       </c>
       <c r="O13" s="101">
         <v>0</v>
       </c>
-      <c r="P13" s="122"/>
-      <c r="Q13" s="120"/>
-    </row>
-    <row r="14" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B14" s="132" t="s">
+      <c r="P13" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R13" s="120"/>
+    </row>
+    <row r="14" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B14" s="131" t="s">
         <v>2</v>
       </c>
       <c r="C14" s="99"/>
       <c r="E14" s="92"/>
       <c r="F14" s="105" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G14" s="106">
         <f>SUM(G5:G13)</f>
@@ -4872,24 +4984,32 @@
         <v>0</v>
       </c>
       <c r="I14" s="103" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J14" s="104">
         <v>0</v>
       </c>
       <c r="K14" s="109"/>
       <c r="M14" s="100"/>
-      <c r="N14" s="53" t="s">
-        <v>41</v>
-      </c>
-      <c r="O14" s="101">
-        <v>0</v>
-      </c>
-      <c r="P14" s="122"/>
-      <c r="Q14" s="120"/>
-    </row>
-    <row r="15" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B15" s="132" t="s">
+      <c r="N14" s="145" t="s">
+        <v>192</v>
+      </c>
+      <c r="O14" s="195">
+        <f>SUM(O5:O13)</f>
+        <v>0</v>
+      </c>
+      <c r="P14" s="195">
+        <f>SUM(P5:P13)</f>
+        <v>0</v>
+      </c>
+      <c r="Q14" s="195">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R14" s="120"/>
+    </row>
+    <row r="15" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B15" s="131" t="s">
         <v>3</v>
       </c>
       <c r="C15" s="99"/>
@@ -4898,7 +5018,7 @@
       <c r="G15" s="94"/>
       <c r="H15" s="95"/>
       <c r="I15" s="103" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J15" s="104">
         <v>0</v>
@@ -4906,25 +5026,31 @@
       <c r="K15" s="109"/>
       <c r="M15" s="100"/>
       <c r="N15" s="53" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="O15" s="101">
         <v>0</v>
       </c>
-      <c r="P15" s="122"/>
-      <c r="Q15" s="120"/>
-    </row>
-    <row r="16" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="132" t="s">
+      <c r="P15" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R15" s="120"/>
+    </row>
+    <row r="16" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B16" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="133"/>
+      <c r="C16" s="132"/>
       <c r="E16" s="92"/>
       <c r="F16" s="93"/>
       <c r="G16" s="93"/>
       <c r="H16" s="93"/>
       <c r="I16" s="103" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J16" s="104">
         <v>0</v>
@@ -4932,17 +5058,23 @@
       <c r="K16" s="119"/>
       <c r="M16" s="100"/>
       <c r="N16" s="53" t="s">
-        <v>45</v>
+        <v>193</v>
       </c>
       <c r="O16" s="101">
         <v>0</v>
       </c>
-      <c r="P16" s="122"/>
-      <c r="Q16" s="120"/>
-    </row>
-    <row r="17" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B17" s="132" t="s">
-        <v>12</v>
+      <c r="P16" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R16" s="120"/>
+    </row>
+    <row r="17" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B17" s="131" t="s">
+        <v>11</v>
       </c>
       <c r="C17" s="99"/>
       <c r="E17" s="92"/>
@@ -4950,7 +5082,7 @@
       <c r="G17" s="93"/>
       <c r="H17" s="93"/>
       <c r="I17" s="103" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J17" s="104">
         <v>0</v>
@@ -4958,43 +5090,57 @@
       <c r="K17" s="119"/>
       <c r="M17" s="100"/>
       <c r="N17" s="53" t="s">
-        <v>184</v>
+        <v>43</v>
       </c>
       <c r="O17" s="101">
         <v>0</v>
       </c>
-      <c r="P17" s="122"/>
-      <c r="Q17" s="120"/>
-    </row>
-    <row r="18" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B18" s="132" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="162"/>
+      <c r="P17" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R17" s="120"/>
+    </row>
+    <row r="18" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B18" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="159"/>
       <c r="E18" s="92"/>
       <c r="F18" s="93"/>
       <c r="G18" s="93"/>
       <c r="H18" s="93"/>
       <c r="I18" s="103" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J18" s="104">
         <v>0</v>
       </c>
       <c r="K18" s="119"/>
       <c r="M18" s="100"/>
-      <c r="N18" s="53" t="s">
-        <v>48</v>
-      </c>
-      <c r="O18" s="101">
-        <v>0</v>
-      </c>
-      <c r="P18" s="122"/>
-      <c r="Q18" s="120"/>
-    </row>
-    <row r="19" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B19" s="132" t="s">
-        <v>23</v>
+      <c r="N18" s="145" t="s">
+        <v>194</v>
+      </c>
+      <c r="O18" s="195">
+        <f>SUM(O15:O17)</f>
+        <v>0</v>
+      </c>
+      <c r="P18" s="195">
+        <f>SUM(P15:P17)</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="195">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R18" s="120"/>
+    </row>
+    <row r="19" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B19" s="131" t="s">
+        <v>22</v>
       </c>
       <c r="C19" s="99"/>
       <c r="E19" s="92"/>
@@ -5002,7 +5148,7 @@
       <c r="G19" s="93"/>
       <c r="H19" s="93"/>
       <c r="I19" s="103" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J19" s="104">
         <v>0</v>
@@ -5010,117 +5156,155 @@
       <c r="K19" s="119"/>
       <c r="M19" s="100"/>
       <c r="N19" s="53" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="O19" s="101">
         <v>0</v>
       </c>
-      <c r="P19" s="122"/>
-      <c r="Q19" s="120"/>
-    </row>
-    <row r="20" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B20" s="135" t="s">
-        <v>176</v>
-      </c>
-      <c r="C20" s="136"/>
+      <c r="P19" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R19" s="120"/>
+    </row>
+    <row r="20" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B20" s="134" t="s">
+        <v>174</v>
+      </c>
+      <c r="C20" s="135"/>
       <c r="E20" s="92"/>
       <c r="F20" s="93"/>
       <c r="G20" s="93"/>
       <c r="H20" s="93"/>
       <c r="I20" s="103" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J20" s="104">
         <v>0</v>
       </c>
       <c r="K20" s="119"/>
       <c r="L20" s="5"/>
-      <c r="M20" s="123"/>
+      <c r="M20" s="122"/>
       <c r="N20" s="53" t="s">
-        <v>52</v>
+        <v>181</v>
       </c>
       <c r="O20" s="101">
         <v>0</v>
       </c>
-      <c r="P20" s="122"/>
-      <c r="Q20" s="120"/>
-    </row>
-    <row r="21" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="137" t="s">
-        <v>163</v>
-      </c>
-      <c r="C21" s="136"/>
+      <c r="P20" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R20" s="120"/>
+    </row>
+    <row r="21" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="136" t="s">
+        <v>161</v>
+      </c>
+      <c r="C21" s="135"/>
       <c r="E21" s="92"/>
       <c r="F21" s="93"/>
       <c r="G21" s="93"/>
       <c r="H21" s="93"/>
       <c r="I21" s="103" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J21" s="104">
         <v>0</v>
       </c>
       <c r="K21" s="119"/>
       <c r="L21" s="5"/>
-      <c r="M21" s="123"/>
+      <c r="M21" s="122"/>
       <c r="N21" s="53" t="s">
-        <v>188</v>
+        <v>46</v>
       </c>
       <c r="O21" s="101">
         <v>0</v>
       </c>
-      <c r="P21" s="122"/>
-      <c r="Q21" s="120"/>
-    </row>
-    <row r="22" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="135" t="s">
-        <v>164</v>
-      </c>
-      <c r="C22" s="136"/>
+      <c r="P21" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R21" s="120"/>
+    </row>
+    <row r="22" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="134" t="s">
+        <v>162</v>
+      </c>
+      <c r="C22" s="135"/>
       <c r="E22" s="92"/>
       <c r="F22" s="93"/>
       <c r="G22" s="93"/>
       <c r="H22" s="93"/>
       <c r="I22" s="103" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J22" s="104">
         <v>0</v>
       </c>
       <c r="K22" s="92"/>
-      <c r="M22" s="148"/>
-      <c r="N22" s="139"/>
-      <c r="O22" s="147"/>
-      <c r="P22" s="147"/>
-      <c r="Q22" s="120"/>
-    </row>
-    <row r="23" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="139"/>
-      <c r="C23" s="139"/>
+      <c r="M22" s="145"/>
+      <c r="N22" s="145" t="s">
+        <v>195</v>
+      </c>
+      <c r="O22" s="195">
+        <f>SUM(O19:O21)</f>
+        <v>0</v>
+      </c>
+      <c r="P22" s="195">
+        <f>SUM(P19:P21)</f>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="195">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R22" s="120"/>
+    </row>
+    <row r="23" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="138"/>
+      <c r="C23" s="138"/>
       <c r="E23" s="92"/>
       <c r="F23" s="93"/>
       <c r="G23" s="93"/>
       <c r="H23" s="93"/>
       <c r="I23" s="107" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J23" s="108">
         <f>SUM(J5:J22)</f>
         <v>0</v>
       </c>
       <c r="K23" s="92"/>
-      <c r="M23" s="148"/>
-      <c r="N23" s="165" t="s">
-        <v>62</v>
-      </c>
-      <c r="O23" s="165"/>
-      <c r="P23" s="165"/>
-      <c r="Q23" s="120"/>
-    </row>
-    <row r="24" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M23" s="145"/>
+      <c r="N23" s="53" t="s">
+        <v>48</v>
+      </c>
+      <c r="O23" s="101">
+        <v>0</v>
+      </c>
+      <c r="P23" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R23" s="120"/>
+    </row>
+    <row r="24" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
-      <c r="B24" s="145" t="s">
-        <v>165</v>
+      <c r="B24" s="142" t="s">
+        <v>163</v>
       </c>
       <c r="C24" s="99"/>
       <c r="D24" s="6"/>
@@ -5132,12 +5316,21 @@
       <c r="J24" s="92"/>
       <c r="K24" s="92"/>
       <c r="L24" s="6"/>
-      <c r="M24" s="124"/>
-      <c r="N24" s="139"/>
-      <c r="O24" s="139"/>
-      <c r="P24" s="139"/>
-      <c r="Q24" s="161"/>
-      <c r="R24" s="6"/>
+      <c r="M24" s="123"/>
+      <c r="N24" s="53" t="s">
+        <v>50</v>
+      </c>
+      <c r="O24" s="101">
+        <v>0</v>
+      </c>
+      <c r="P24" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R24" s="158"/>
       <c r="S24" s="6"/>
       <c r="T24" s="6"/>
       <c r="U24" s="6"/>
@@ -5146,39 +5339,46 @@
       <c r="X24" s="6"/>
       <c r="Y24" s="6"/>
       <c r="Z24" s="6"/>
-    </row>
-    <row r="25" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="134" t="s">
-        <v>166</v>
+      <c r="AA24" s="6"/>
+    </row>
+    <row r="25" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="133" t="s">
+        <v>164</v>
       </c>
       <c r="C25" s="99"/>
       <c r="E25" s="109"/>
-      <c r="F25" s="168" t="s">
-        <v>54</v>
-      </c>
-      <c r="G25" s="169"/>
-      <c r="H25" s="169"/>
-      <c r="I25" s="169"/>
+      <c r="F25" s="165" t="s">
+        <v>52</v>
+      </c>
+      <c r="G25" s="166"/>
+      <c r="H25" s="166"/>
+      <c r="I25" s="166"/>
       <c r="J25" s="110">
         <f>SUM(G14:H14)-J23</f>
         <v>0</v>
       </c>
       <c r="K25" s="109"/>
-      <c r="M25" s="124"/>
-      <c r="N25" s="125" t="s">
-        <v>66</v>
-      </c>
-      <c r="O25" s="125" t="s">
-        <v>7</v>
-      </c>
-      <c r="P25" s="125"/>
-      <c r="Q25" s="120"/>
-    </row>
-    <row r="26" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="135" t="s">
-        <v>181</v>
-      </c>
-      <c r="C26" s="136"/>
+      <c r="M25" s="123"/>
+      <c r="N25" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="O25" s="101">
+        <v>0</v>
+      </c>
+      <c r="P25" s="101">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="101">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R25" s="120"/>
+    </row>
+    <row r="26" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="134" t="s">
+        <v>178</v>
+      </c>
+      <c r="C26" s="135"/>
       <c r="E26" s="92"/>
       <c r="F26" s="92"/>
       <c r="G26" s="94"/>
@@ -5186,21 +5386,29 @@
       <c r="I26" s="92"/>
       <c r="J26" s="92"/>
       <c r="K26" s="92"/>
-      <c r="M26" s="124"/>
-      <c r="N26" s="53" t="s">
-        <v>69</v>
-      </c>
-      <c r="O26" s="101">
-        <v>0</v>
-      </c>
-      <c r="P26" s="101"/>
-      <c r="Q26" s="120"/>
-    </row>
-    <row r="27" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="135" t="s">
-        <v>182</v>
-      </c>
-      <c r="C27" s="136"/>
+      <c r="M26" s="123"/>
+      <c r="N26" s="145" t="s">
+        <v>197</v>
+      </c>
+      <c r="O26" s="195">
+        <f>SUM(O23:O25)</f>
+        <v>0</v>
+      </c>
+      <c r="P26" s="195">
+        <f>SUM(P23:P25)</f>
+        <v>0</v>
+      </c>
+      <c r="Q26" s="195">
+        <f t="shared" ref="Q26" si="1">SUM(O26:P26)</f>
+        <v>0</v>
+      </c>
+      <c r="R26" s="120"/>
+    </row>
+    <row r="27" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="134" t="s">
+        <v>179</v>
+      </c>
+      <c r="C27" s="135"/>
       <c r="E27" s="92"/>
       <c r="F27" s="92"/>
       <c r="G27" s="94"/>
@@ -5208,214 +5416,229 @@
       <c r="I27" s="92"/>
       <c r="J27" s="92"/>
       <c r="K27" s="92"/>
-      <c r="M27" s="124"/>
-      <c r="N27" s="126" t="s">
-        <v>70</v>
-      </c>
-      <c r="O27" s="101">
-        <v>0</v>
-      </c>
-      <c r="P27" s="101"/>
-      <c r="Q27" s="120"/>
-    </row>
-    <row r="28" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="135" t="s">
-        <v>183</v>
-      </c>
-      <c r="C28" s="136"/>
+      <c r="M27" s="123"/>
+      <c r="N27" s="196" t="s">
+        <v>38</v>
+      </c>
+      <c r="O27" s="197">
+        <f>O14+O18+O22+O26</f>
+        <v>0</v>
+      </c>
+      <c r="P27" s="197">
+        <f t="shared" ref="P27:Q27" si="2">P14+P18+P22+P26</f>
+        <v>0</v>
+      </c>
+      <c r="Q27" s="197">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R27" s="120"/>
+    </row>
+    <row r="28" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="134" t="s">
+        <v>180</v>
+      </c>
+      <c r="C28" s="135"/>
       <c r="E28" s="92"/>
-      <c r="F28" s="166" t="s">
-        <v>55</v>
-      </c>
-      <c r="G28" s="167"/>
+      <c r="F28" s="163" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28" s="164"/>
       <c r="H28" s="95"/>
-      <c r="I28" s="176" t="s">
-        <v>56</v>
-      </c>
-      <c r="J28" s="177"/>
+      <c r="I28" s="173" t="s">
+        <v>54</v>
+      </c>
+      <c r="J28" s="174"/>
       <c r="K28" s="92"/>
       <c r="M28" s="100"/>
-      <c r="N28" s="53" t="s">
-        <v>71</v>
-      </c>
-      <c r="O28" s="101">
-        <v>0</v>
-      </c>
-      <c r="P28" s="101"/>
-      <c r="Q28" s="120"/>
-    </row>
-    <row r="29" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="139"/>
-      <c r="C29" s="139"/>
+      <c r="N28" s="138"/>
+      <c r="O28" s="144"/>
+      <c r="P28" s="144"/>
+      <c r="Q28" s="144"/>
+      <c r="R28" s="120"/>
+    </row>
+    <row r="29" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="138"/>
+      <c r="C29" s="138"/>
       <c r="E29" s="92"/>
       <c r="F29" s="103" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G29" s="112">
         <v>0</v>
       </c>
       <c r="H29" s="95"/>
       <c r="I29" s="113" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="J29" s="114">
         <v>0</v>
       </c>
       <c r="K29" s="92"/>
-      <c r="M29" s="148"/>
-      <c r="N29" s="53" t="s">
-        <v>73</v>
-      </c>
-      <c r="O29" s="101">
-        <v>0</v>
-      </c>
-      <c r="P29" s="101"/>
-      <c r="Q29" s="93"/>
-    </row>
-    <row r="30" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="146" t="s">
-        <v>170</v>
-      </c>
-      <c r="C30" s="138"/>
+      <c r="M29" s="145"/>
+      <c r="N29" s="162" t="s">
+        <v>60</v>
+      </c>
+      <c r="O29" s="162"/>
+      <c r="P29" s="162"/>
+      <c r="Q29" s="144"/>
+      <c r="R29" s="93"/>
+    </row>
+    <row r="30" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="143" t="s">
+        <v>168</v>
+      </c>
+      <c r="C30" s="137"/>
       <c r="E30" s="92"/>
       <c r="F30" s="103" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G30" s="112">
         <v>0</v>
       </c>
       <c r="H30" s="95"/>
       <c r="I30" s="113" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J30" s="114">
         <v>0</v>
       </c>
       <c r="K30" s="92"/>
-      <c r="M30" s="139"/>
-      <c r="N30" s="53" t="s">
-        <v>74</v>
-      </c>
-      <c r="O30" s="101">
-        <v>0</v>
-      </c>
-      <c r="P30" s="101"/>
-      <c r="Q30" s="139"/>
-    </row>
-    <row r="31" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="135" t="s">
-        <v>178</v>
-      </c>
-      <c r="C31" s="136"/>
+      <c r="M30" s="138"/>
+      <c r="N30" s="138"/>
+      <c r="O30" s="138"/>
+      <c r="P30" s="138"/>
+      <c r="Q30" s="138"/>
+      <c r="R30" s="138"/>
+    </row>
+    <row r="31" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="134" t="s">
+        <v>202</v>
+      </c>
+      <c r="C31" s="135"/>
       <c r="E31" s="92"/>
       <c r="F31" s="113" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G31" s="112">
         <v>0</v>
       </c>
       <c r="H31" s="95"/>
       <c r="I31" s="113" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J31" s="114">
         <v>0</v>
       </c>
       <c r="K31" s="92"/>
       <c r="M31" s="92"/>
-      <c r="N31" s="139"/>
-      <c r="O31" s="139"/>
-      <c r="P31" s="139"/>
-      <c r="Q31" s="93"/>
-    </row>
-    <row r="32" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="140"/>
+      <c r="N31" s="124" t="s">
+        <v>64</v>
+      </c>
+      <c r="O31" s="124" t="s">
+        <v>7</v>
+      </c>
+      <c r="P31" s="124"/>
+      <c r="Q31" s="124"/>
+      <c r="R31" s="93"/>
+    </row>
+    <row r="32" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="134" t="s">
+        <v>200</v>
+      </c>
       <c r="C32" s="99"/>
       <c r="E32" s="92"/>
       <c r="F32" s="103" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G32" s="112">
         <v>0</v>
       </c>
       <c r="H32" s="95"/>
       <c r="I32" s="113" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="J32" s="114">
         <v>0</v>
       </c>
       <c r="K32" s="92"/>
       <c r="M32" s="92"/>
-      <c r="N32" s="125" t="s">
-        <v>177</v>
-      </c>
-      <c r="O32" s="125" t="s">
-        <v>171</v>
-      </c>
-      <c r="P32" s="125" t="s">
-        <v>172</v>
-      </c>
-      <c r="Q32" s="120"/>
-    </row>
-    <row r="33" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="143"/>
-      <c r="C33" s="144"/>
+      <c r="N32" s="53" t="s">
+        <v>67</v>
+      </c>
+      <c r="O32" s="101">
+        <v>0</v>
+      </c>
+      <c r="P32" s="101"/>
+      <c r="Q32" s="101"/>
+      <c r="R32" s="120"/>
+    </row>
+    <row r="33" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="200" t="s">
+        <v>201</v>
+      </c>
+      <c r="C33" s="141"/>
       <c r="E33" s="92"/>
       <c r="F33" s="103" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G33" s="112">
         <v>0</v>
       </c>
       <c r="H33" s="95"/>
       <c r="I33" s="113" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J33" s="114">
         <v>0</v>
       </c>
       <c r="K33" s="92"/>
       <c r="M33" s="92"/>
-      <c r="N33" s="127" t="s">
-        <v>173</v>
-      </c>
-      <c r="O33" s="128"/>
-      <c r="P33" s="129"/>
-      <c r="Q33" s="120"/>
-    </row>
-    <row r="34" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="139"/>
-      <c r="C34" s="139"/>
+      <c r="N33" s="125" t="s">
+        <v>68</v>
+      </c>
+      <c r="O33" s="101">
+        <v>0</v>
+      </c>
+      <c r="P33" s="101"/>
+      <c r="Q33" s="101"/>
+      <c r="R33" s="120"/>
+    </row>
+    <row r="34" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="138"/>
+      <c r="C34" s="138"/>
       <c r="E34" s="92"/>
       <c r="F34" s="103" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G34" s="112">
         <v>0</v>
       </c>
       <c r="H34" s="95"/>
       <c r="I34" s="113" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="J34" s="114">
         <v>0</v>
       </c>
       <c r="K34" s="92"/>
       <c r="M34" s="92"/>
-      <c r="N34" s="127" t="s">
-        <v>174</v>
-      </c>
-      <c r="O34" s="129"/>
-      <c r="P34" s="129"/>
-      <c r="Q34" s="120"/>
-    </row>
-    <row r="35" spans="2:18" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B35" s="139"/>
-      <c r="C35" s="139"/>
+      <c r="N34" s="53" t="s">
+        <v>69</v>
+      </c>
+      <c r="O34" s="101">
+        <v>0</v>
+      </c>
+      <c r="P34" s="101"/>
+      <c r="Q34" s="101"/>
+      <c r="R34" s="120"/>
+    </row>
+    <row r="35" spans="2:19" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B35" s="138"/>
+      <c r="C35" s="138"/>
       <c r="E35" s="92"/>
       <c r="F35" s="115" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G35" s="116">
         <f>SUM(G29:G34)</f>
@@ -5423,7 +5646,7 @@
       </c>
       <c r="H35" s="95"/>
       <c r="I35" s="111" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J35" s="117">
         <f>SUM(J29:J34)</f>
@@ -5431,14 +5654,17 @@
       </c>
       <c r="K35" s="92"/>
       <c r="M35" s="92"/>
-      <c r="N35" s="127" t="s">
-        <v>179</v>
-      </c>
-      <c r="O35" s="129"/>
-      <c r="P35" s="129"/>
-      <c r="Q35" s="120"/>
-    </row>
-    <row r="36" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N35" s="53" t="s">
+        <v>71</v>
+      </c>
+      <c r="O35" s="101">
+        <v>0</v>
+      </c>
+      <c r="P35" s="101"/>
+      <c r="Q35" s="101"/>
+      <c r="R35" s="120"/>
+    </row>
+    <row r="36" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="93"/>
       <c r="C36" s="99"/>
       <c r="E36" s="92"/>
@@ -5449,57 +5675,64 @@
       <c r="J36" s="95"/>
       <c r="K36" s="92"/>
       <c r="M36" s="92"/>
-      <c r="N36" s="127" t="s">
-        <v>180</v>
-      </c>
-      <c r="O36" s="130"/>
-      <c r="P36" s="129"/>
-      <c r="Q36" s="120"/>
-    </row>
-    <row r="37" spans="2:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="139"/>
-      <c r="C37" s="139"/>
+      <c r="N36" s="53" t="s">
+        <v>72</v>
+      </c>
+      <c r="O36" s="101">
+        <v>0</v>
+      </c>
+      <c r="P36" s="101"/>
+      <c r="Q36" s="101"/>
+      <c r="R36" s="120"/>
+    </row>
+    <row r="37" spans="2:19" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="93"/>
+      <c r="C37" s="99"/>
       <c r="E37" s="92"/>
-      <c r="F37" s="168" t="s">
-        <v>72</v>
-      </c>
-      <c r="G37" s="169"/>
-      <c r="H37" s="110">
-        <f>J25-J35-G35</f>
-        <v>0</v>
-      </c>
-      <c r="I37" s="92"/>
-      <c r="J37" s="92"/>
+      <c r="F37" s="92"/>
+      <c r="G37" s="94"/>
+      <c r="H37" s="95"/>
+      <c r="I37" s="95"/>
+      <c r="J37" s="95"/>
       <c r="K37" s="92"/>
       <c r="M37" s="92"/>
-      <c r="N37" s="127" t="s">
-        <v>175</v>
-      </c>
-      <c r="O37" s="131"/>
-      <c r="P37" s="129"/>
-      <c r="Q37" s="120"/>
-    </row>
-    <row r="38" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="139"/>
-      <c r="C38" s="139"/>
+      <c r="N37" s="138"/>
+      <c r="O37" s="138"/>
+      <c r="P37" s="138"/>
+      <c r="Q37" s="138"/>
+      <c r="R37" s="120"/>
+    </row>
+    <row r="38" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="138"/>
+      <c r="C38" s="138"/>
       <c r="E38" s="92"/>
-      <c r="F38" s="96"/>
-      <c r="G38" s="97"/>
-      <c r="H38" s="95"/>
-      <c r="I38" s="92"/>
-      <c r="J38" s="92"/>
+      <c r="F38" s="165" t="s">
+        <v>70</v>
+      </c>
+      <c r="G38" s="165"/>
+      <c r="H38" s="165"/>
+      <c r="I38" s="165"/>
+      <c r="J38" s="110">
+        <f>J25-J35</f>
+        <v>0</v>
+      </c>
       <c r="K38" s="92"/>
       <c r="M38" s="92"/>
-      <c r="N38" s="127" t="s">
-        <v>185</v>
-      </c>
-      <c r="O38" s="131"/>
-      <c r="P38" s="129"/>
-      <c r="Q38" s="120"/>
-    </row>
-    <row r="39" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="139"/>
-      <c r="C39" s="139"/>
+      <c r="N38" s="124" t="s">
+        <v>175</v>
+      </c>
+      <c r="O38" s="124" t="s">
+        <v>169</v>
+      </c>
+      <c r="P38" s="124" t="s">
+        <v>170</v>
+      </c>
+      <c r="Q38" s="124"/>
+      <c r="R38" s="120"/>
+    </row>
+    <row r="39" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="138"/>
+      <c r="C39" s="138"/>
       <c r="E39" s="92"/>
       <c r="F39" s="96"/>
       <c r="G39" s="97"/>
@@ -5508,243 +5741,327 @@
       <c r="J39" s="92"/>
       <c r="K39" s="92"/>
       <c r="M39" s="92"/>
-      <c r="N39" s="139"/>
-      <c r="O39" s="139"/>
-      <c r="P39" s="139"/>
-      <c r="Q39" s="120"/>
-    </row>
-    <row r="40" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="135"/>
-      <c r="C40" s="136"/>
+      <c r="N39" s="126" t="s">
+        <v>171</v>
+      </c>
+      <c r="O39" s="127"/>
+      <c r="P39" s="128"/>
+      <c r="Q39" s="128"/>
+      <c r="R39" s="120"/>
+    </row>
+    <row r="40" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="138"/>
+      <c r="C40" s="138"/>
       <c r="E40" s="92"/>
-      <c r="F40" s="96"/>
-      <c r="G40" s="97"/>
-      <c r="H40" s="98" t="s">
-        <v>75</v>
-      </c>
-      <c r="I40" s="92"/>
-      <c r="J40" s="92"/>
+      <c r="F40" s="165" t="s">
+        <v>198</v>
+      </c>
+      <c r="G40" s="165"/>
+      <c r="H40" s="165"/>
+      <c r="I40" s="165"/>
+      <c r="J40" s="110">
+        <f>J25-J35-G35</f>
+        <v>0</v>
+      </c>
       <c r="K40" s="92"/>
       <c r="M40" s="92"/>
-      <c r="N40" s="139"/>
-      <c r="O40" s="139"/>
-      <c r="P40" s="139"/>
-      <c r="Q40" s="120"/>
-    </row>
-    <row r="41" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="150"/>
-      <c r="C41" s="150"/>
-      <c r="D41" s="150"/>
-      <c r="E41" s="151"/>
-      <c r="F41" s="152"/>
-      <c r="G41" s="153"/>
-      <c r="H41" s="154"/>
-      <c r="I41" s="151"/>
-      <c r="J41" s="151"/>
-      <c r="K41" s="151"/>
-      <c r="L41" s="150"/>
-      <c r="M41" s="151"/>
-      <c r="N41" s="150"/>
-      <c r="O41" s="150"/>
-      <c r="P41" s="150"/>
-      <c r="Q41" s="149"/>
-      <c r="R41" s="150"/>
-    </row>
-    <row r="42" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="150"/>
-      <c r="C42" s="150"/>
-      <c r="D42" s="150"/>
-      <c r="E42" s="151"/>
-      <c r="F42" s="152"/>
-      <c r="G42" s="153"/>
-      <c r="H42" s="154"/>
-      <c r="I42" s="151"/>
-      <c r="J42" s="151"/>
-      <c r="K42" s="151"/>
-      <c r="L42" s="150"/>
-      <c r="M42" s="151"/>
-      <c r="N42" s="150"/>
-      <c r="O42" s="150"/>
-      <c r="P42" s="150"/>
-      <c r="Q42" s="149"/>
-      <c r="R42" s="150"/>
-    </row>
-    <row r="43" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="150"/>
-      <c r="C43" s="150"/>
-      <c r="D43" s="150"/>
-      <c r="E43" s="151"/>
-      <c r="F43" s="152"/>
-      <c r="G43" s="153"/>
-      <c r="H43" s="154"/>
-      <c r="I43" s="151"/>
-      <c r="J43" s="151"/>
-      <c r="K43" s="151"/>
-      <c r="L43" s="150"/>
-      <c r="M43" s="151"/>
-      <c r="N43" s="150"/>
-      <c r="O43" s="150"/>
-      <c r="P43" s="150"/>
-      <c r="Q43" s="149"/>
-      <c r="R43" s="150"/>
-    </row>
-    <row r="44" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="150"/>
-      <c r="C44" s="150"/>
-      <c r="D44" s="150"/>
-      <c r="E44" s="151"/>
-      <c r="F44" s="149"/>
-      <c r="G44" s="155"/>
-      <c r="H44" s="156"/>
-      <c r="I44" s="155"/>
-      <c r="J44" s="155"/>
-      <c r="K44" s="151"/>
-      <c r="L44" s="150"/>
-      <c r="M44" s="149"/>
-      <c r="N44" s="150"/>
-      <c r="O44" s="150"/>
-      <c r="P44" s="150"/>
-      <c r="Q44" s="149"/>
-      <c r="R44" s="150"/>
-    </row>
-    <row r="45" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="149"/>
-      <c r="C45" s="157"/>
-      <c r="D45" s="150"/>
-      <c r="E45" s="149"/>
-      <c r="F45" s="149"/>
-      <c r="G45" s="158"/>
-      <c r="H45" s="157"/>
-      <c r="I45" s="149"/>
-      <c r="J45" s="149"/>
-      <c r="K45" s="149"/>
-      <c r="L45" s="150"/>
-      <c r="M45" s="149"/>
-      <c r="N45" s="150"/>
-      <c r="O45" s="150"/>
-      <c r="P45" s="150"/>
-      <c r="Q45" s="149"/>
-      <c r="R45" s="150"/>
-    </row>
-    <row r="46" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="149"/>
-      <c r="C46" s="157"/>
-      <c r="D46" s="150"/>
-      <c r="E46" s="149"/>
-      <c r="F46" s="155"/>
-      <c r="G46" s="155"/>
-      <c r="H46" s="150"/>
-      <c r="I46" s="155"/>
-      <c r="J46" s="149"/>
-      <c r="K46" s="149"/>
-      <c r="L46" s="150"/>
-      <c r="M46" s="149"/>
-      <c r="N46" s="149"/>
-      <c r="O46" s="149"/>
-      <c r="P46" s="149"/>
-      <c r="Q46" s="149"/>
-      <c r="R46" s="150"/>
-    </row>
-    <row r="47" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="150"/>
-      <c r="C47" s="159"/>
-      <c r="D47" s="150"/>
-      <c r="E47" s="150"/>
-      <c r="F47" s="150"/>
-      <c r="G47" s="160"/>
-      <c r="H47" s="159"/>
-      <c r="I47" s="150"/>
-      <c r="J47" s="150"/>
-      <c r="K47" s="150"/>
-      <c r="L47" s="150"/>
-      <c r="M47" s="150"/>
-      <c r="N47" s="150"/>
-      <c r="O47" s="150"/>
-      <c r="P47" s="150"/>
-      <c r="Q47" s="150"/>
-      <c r="R47" s="150"/>
-    </row>
-    <row r="48" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C48" s="1"/>
-      <c r="G48" s="3"/>
-      <c r="H48" s="1"/>
-    </row>
-    <row r="49" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C49" s="1"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="1"/>
-    </row>
-    <row r="50" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C50" s="1"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="1"/>
-    </row>
-    <row r="51" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C51" s="1"/>
-      <c r="G51" s="3"/>
-      <c r="H51" s="1"/>
-    </row>
-    <row r="52" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C52" s="1"/>
-      <c r="G52" s="3"/>
-      <c r="H52" s="1"/>
-    </row>
-    <row r="53" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N40" s="126" t="s">
+        <v>172</v>
+      </c>
+      <c r="O40" s="128"/>
+      <c r="P40" s="128"/>
+      <c r="Q40" s="128"/>
+      <c r="R40" s="120"/>
+    </row>
+    <row r="41" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="138"/>
+      <c r="C41" s="138"/>
+      <c r="E41" s="92"/>
+      <c r="F41" s="92"/>
+      <c r="G41" s="92"/>
+      <c r="H41" s="92"/>
+      <c r="I41" s="92"/>
+      <c r="J41" s="92"/>
+      <c r="K41" s="92"/>
+      <c r="L41" s="147"/>
+      <c r="M41" s="92"/>
+      <c r="N41" s="126" t="s">
+        <v>176</v>
+      </c>
+      <c r="O41" s="128"/>
+      <c r="P41" s="128"/>
+      <c r="Q41" s="128"/>
+      <c r="R41" s="120"/>
+      <c r="S41" s="147"/>
+    </row>
+    <row r="42" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="138"/>
+      <c r="C42" s="138"/>
+      <c r="E42" s="92"/>
+      <c r="F42" s="199" t="s">
+        <v>199</v>
+      </c>
+      <c r="G42" s="199"/>
+      <c r="H42" s="199"/>
+      <c r="I42" s="199"/>
+      <c r="J42" s="198">
+        <v>0</v>
+      </c>
+      <c r="K42" s="92"/>
+      <c r="L42" s="147"/>
+      <c r="M42" s="92"/>
+      <c r="N42" s="126" t="s">
+        <v>177</v>
+      </c>
+      <c r="O42" s="129"/>
+      <c r="P42" s="128"/>
+      <c r="Q42" s="128"/>
+      <c r="R42" s="120"/>
+      <c r="S42" s="147"/>
+    </row>
+    <row r="43" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="138"/>
+      <c r="C43" s="138"/>
+      <c r="E43" s="92"/>
+      <c r="F43" s="199"/>
+      <c r="G43" s="199"/>
+      <c r="H43" s="199"/>
+      <c r="I43" s="199"/>
+      <c r="J43" s="198"/>
+      <c r="K43" s="92"/>
+      <c r="L43" s="147"/>
+      <c r="M43" s="92"/>
+      <c r="N43" s="126" t="s">
+        <v>173</v>
+      </c>
+      <c r="O43" s="130"/>
+      <c r="P43" s="128"/>
+      <c r="Q43" s="128"/>
+      <c r="R43" s="120"/>
+      <c r="S43" s="147"/>
+    </row>
+    <row r="44" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="138"/>
+      <c r="C44" s="138"/>
+      <c r="E44" s="92"/>
+      <c r="F44" s="96"/>
+      <c r="G44" s="97"/>
+      <c r="H44" s="95"/>
+      <c r="I44" s="92"/>
+      <c r="J44" s="92"/>
+      <c r="K44" s="92"/>
+      <c r="L44" s="147"/>
+      <c r="M44" s="92"/>
+      <c r="N44" s="126" t="s">
+        <v>182</v>
+      </c>
+      <c r="O44" s="130"/>
+      <c r="P44" s="128"/>
+      <c r="Q44" s="128"/>
+      <c r="R44" s="120"/>
+      <c r="S44" s="147"/>
+    </row>
+    <row r="45" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="134"/>
+      <c r="C45" s="135"/>
+      <c r="E45" s="92"/>
+      <c r="F45" s="96"/>
+      <c r="G45" s="97"/>
+      <c r="H45" s="98" t="s">
+        <v>73</v>
+      </c>
+      <c r="I45" s="92"/>
+      <c r="J45" s="92"/>
+      <c r="K45" s="92"/>
+      <c r="L45" s="147"/>
+      <c r="M45" s="92"/>
+      <c r="N45" s="138"/>
+      <c r="O45" s="138"/>
+      <c r="P45" s="138"/>
+      <c r="Q45" s="138"/>
+      <c r="R45" s="120"/>
+      <c r="S45" s="147"/>
+    </row>
+    <row r="46" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="147"/>
+      <c r="C46" s="147"/>
+      <c r="D46" s="147"/>
+      <c r="E46" s="148"/>
+      <c r="F46" s="149"/>
+      <c r="G46" s="150"/>
+      <c r="H46" s="151"/>
+      <c r="I46" s="148"/>
+      <c r="J46" s="148"/>
+      <c r="K46" s="148"/>
+      <c r="L46" s="146"/>
+      <c r="M46" s="146"/>
+      <c r="N46" s="146"/>
+      <c r="O46" s="146"/>
+      <c r="P46" s="146"/>
+      <c r="Q46" s="146"/>
+      <c r="R46" s="146"/>
+      <c r="S46" s="147"/>
+    </row>
+    <row r="47" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="147"/>
+      <c r="C47" s="147"/>
+      <c r="D47" s="147"/>
+      <c r="E47" s="148"/>
+      <c r="F47" s="149"/>
+      <c r="G47" s="150"/>
+      <c r="H47" s="151"/>
+      <c r="I47" s="148"/>
+      <c r="J47" s="148"/>
+      <c r="K47" s="148"/>
+      <c r="L47" s="147"/>
+      <c r="M47" s="147"/>
+      <c r="N47" s="147"/>
+      <c r="O47" s="147"/>
+      <c r="P47" s="147"/>
+      <c r="Q47" s="147"/>
+      <c r="R47" s="147"/>
+      <c r="S47" s="147"/>
+    </row>
+    <row r="48" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B48" s="147"/>
+      <c r="C48" s="147"/>
+      <c r="D48" s="147"/>
+      <c r="E48" s="148"/>
+      <c r="F48" s="149"/>
+      <c r="G48" s="150"/>
+      <c r="H48" s="151"/>
+      <c r="I48" s="146"/>
+      <c r="J48" s="146"/>
+      <c r="K48" s="146"/>
+      <c r="N48" s="147"/>
+      <c r="O48" s="147"/>
+      <c r="P48" s="147"/>
+      <c r="Q48" s="147"/>
+    </row>
+    <row r="49" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="147"/>
+      <c r="C49" s="147"/>
+      <c r="D49" s="147"/>
+      <c r="E49" s="148"/>
+      <c r="F49" s="146"/>
+      <c r="G49" s="152"/>
+      <c r="H49" s="153"/>
+      <c r="I49" s="152"/>
+      <c r="J49" s="152"/>
+      <c r="K49" s="148"/>
+      <c r="N49" s="147"/>
+      <c r="O49" s="147"/>
+      <c r="P49" s="147"/>
+      <c r="Q49" s="147"/>
+    </row>
+    <row r="50" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B50" s="146"/>
+      <c r="C50" s="154"/>
+      <c r="D50" s="147"/>
+      <c r="E50" s="146"/>
+      <c r="F50" s="146"/>
+      <c r="G50" s="155"/>
+      <c r="H50" s="154"/>
+      <c r="I50" s="146"/>
+      <c r="J50" s="146"/>
+      <c r="K50" s="146"/>
+      <c r="N50" s="147"/>
+      <c r="O50" s="147"/>
+      <c r="P50" s="147"/>
+      <c r="Q50" s="147"/>
+    </row>
+    <row r="51" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="146"/>
+      <c r="C51" s="154"/>
+      <c r="D51" s="147"/>
+      <c r="E51" s="146"/>
+      <c r="F51" s="152"/>
+      <c r="G51" s="152"/>
+      <c r="H51" s="147"/>
+      <c r="I51" s="152"/>
+      <c r="J51" s="146"/>
+      <c r="K51" s="146"/>
+      <c r="N51" s="147"/>
+      <c r="O51" s="147"/>
+      <c r="P51" s="147"/>
+      <c r="Q51" s="147"/>
+    </row>
+    <row r="52" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="147"/>
+      <c r="C52" s="156"/>
+      <c r="D52" s="147"/>
+      <c r="E52" s="147"/>
+      <c r="F52" s="147"/>
+      <c r="G52" s="157"/>
+      <c r="H52" s="156"/>
+      <c r="I52" s="147"/>
+      <c r="J52" s="147"/>
+      <c r="K52" s="147"/>
+      <c r="N52" s="146"/>
+      <c r="O52" s="146"/>
+      <c r="P52" s="146"/>
+      <c r="Q52" s="146"/>
+    </row>
+    <row r="53" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C53" s="1"/>
       <c r="G53" s="3"/>
       <c r="H53" s="1"/>
-    </row>
-    <row r="54" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N53" s="147"/>
+      <c r="O53" s="147"/>
+      <c r="P53" s="147"/>
+      <c r="Q53" s="147"/>
+    </row>
+    <row r="54" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C54" s="1"/>
       <c r="G54" s="3"/>
       <c r="H54" s="1"/>
     </row>
-    <row r="55" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C55" s="1"/>
       <c r="G55" s="3"/>
       <c r="H55" s="1"/>
     </row>
-    <row r="56" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C56" s="1"/>
       <c r="G56" s="3"/>
       <c r="H56" s="1"/>
     </row>
-    <row r="57" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C57" s="1"/>
       <c r="G57" s="3"/>
       <c r="H57" s="1"/>
     </row>
-    <row r="58" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C58" s="1"/>
       <c r="G58" s="3"/>
       <c r="H58" s="1"/>
     </row>
-    <row r="59" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C59" s="1"/>
       <c r="G59" s="3"/>
       <c r="H59" s="1"/>
     </row>
-    <row r="60" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C60" s="1"/>
       <c r="G60" s="3"/>
       <c r="H60" s="1"/>
     </row>
-    <row r="61" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C61" s="1"/>
       <c r="G61" s="3"/>
       <c r="H61" s="1"/>
     </row>
-    <row r="62" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C62" s="1"/>
       <c r="G62" s="3"/>
       <c r="H62" s="1"/>
     </row>
-    <row r="63" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C63" s="1"/>
       <c r="G63" s="3"/>
       <c r="H63" s="1"/>
     </row>
-    <row r="64" spans="3:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C64" s="1"/>
       <c r="G64" s="3"/>
       <c r="H64" s="1"/>
@@ -10449,13 +10766,40 @@
       <c r="G1004" s="3"/>
       <c r="H1004" s="1"/>
     </row>
+    <row r="1005" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C1005" s="1"/>
+      <c r="G1005" s="3"/>
+      <c r="H1005" s="1"/>
+    </row>
+    <row r="1006" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C1006" s="1"/>
+      <c r="G1006" s="3"/>
+      <c r="H1006" s="1"/>
+    </row>
+    <row r="1007" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C1007" s="1"/>
+      <c r="G1007" s="3"/>
+      <c r="H1007" s="1"/>
+    </row>
+    <row r="1008" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C1008" s="1"/>
+      <c r="G1008" s="3"/>
+      <c r="H1008" s="1"/>
+    </row>
+    <row r="1009" spans="3:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C1009" s="1"/>
+      <c r="G1009" s="3"/>
+      <c r="H1009" s="1"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="O4:P4"/>
+  <mergeCells count="12">
+    <mergeCell ref="J42:J43"/>
+    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="F42:I43"/>
     <mergeCell ref="N2:P2"/>
-    <mergeCell ref="N23:P23"/>
+    <mergeCell ref="N29:P29"/>
     <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F37:G37"/>
     <mergeCell ref="F2:J2"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="I4:J4"/>
@@ -10510,36 +10854,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:30" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C2" s="178" t="s">
+      <c r="C2" s="188" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="189"/>
+      <c r="E2" s="189"/>
+      <c r="F2" s="190"/>
+      <c r="H2" s="188" t="s">
+        <v>75</v>
+      </c>
+      <c r="I2" s="189"/>
+      <c r="J2" s="189"/>
+      <c r="K2" s="190"/>
+      <c r="M2" s="188" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="180"/>
-      <c r="H2" s="178" t="s">
+      <c r="N2" s="189"/>
+      <c r="O2" s="189"/>
+      <c r="P2" s="190"/>
+      <c r="V2" s="191" t="s">
         <v>77</v>
       </c>
-      <c r="I2" s="179"/>
-      <c r="J2" s="179"/>
-      <c r="K2" s="180"/>
-      <c r="M2" s="178" t="s">
+      <c r="W2" s="189"/>
+      <c r="X2" s="189"/>
+      <c r="Y2" s="190"/>
+      <c r="AA2" s="191" t="s">
         <v>78</v>
       </c>
-      <c r="N2" s="179"/>
-      <c r="O2" s="179"/>
-      <c r="P2" s="180"/>
-      <c r="V2" s="181" t="s">
-        <v>79</v>
-      </c>
-      <c r="W2" s="179"/>
-      <c r="X2" s="179"/>
-      <c r="Y2" s="180"/>
-      <c r="AA2" s="181" t="s">
-        <v>80</v>
-      </c>
-      <c r="AB2" s="179"/>
-      <c r="AC2" s="179"/>
-      <c r="AD2" s="180"/>
+      <c r="AB2" s="189"/>
+      <c r="AC2" s="189"/>
+      <c r="AD2" s="190"/>
     </row>
     <row r="3" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C3" s="7"/>
@@ -10566,39 +10910,39 @@
     <row r="4" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C4" s="7"/>
       <c r="D4" s="182" t="s">
-        <v>81</v>
-      </c>
-      <c r="E4" s="183"/>
+        <v>79</v>
+      </c>
+      <c r="E4" s="177"/>
       <c r="F4" s="8"/>
       <c r="H4" s="7"/>
       <c r="I4" s="182" t="s">
-        <v>82</v>
-      </c>
-      <c r="J4" s="183"/>
+        <v>80</v>
+      </c>
+      <c r="J4" s="177"/>
       <c r="K4" s="8"/>
       <c r="M4" s="7"/>
       <c r="N4" s="182" t="s">
-        <v>83</v>
-      </c>
-      <c r="O4" s="183"/>
+        <v>81</v>
+      </c>
+      <c r="O4" s="177"/>
       <c r="P4" s="8"/>
       <c r="V4" s="12"/>
-      <c r="W4" s="184" t="s">
-        <v>84</v>
-      </c>
-      <c r="X4" s="183"/>
+      <c r="W4" s="181" t="s">
+        <v>82</v>
+      </c>
+      <c r="X4" s="177"/>
       <c r="Y4" s="13"/>
       <c r="AA4" s="12"/>
-      <c r="AB4" s="184" t="s">
-        <v>81</v>
-      </c>
-      <c r="AC4" s="183"/>
+      <c r="AB4" s="181" t="s">
+        <v>79</v>
+      </c>
+      <c r="AC4" s="177"/>
       <c r="AD4" s="13"/>
     </row>
     <row r="5" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C5" s="7"/>
       <c r="D5" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E5" s="15">
         <f>SUM('Plan de charge'!O5:O7)</f>
@@ -10608,17 +10952,17 @@
       <c r="G5" s="16"/>
       <c r="H5" s="7"/>
       <c r="I5" s="17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J5" s="18">
-        <f>'Plan de charge'!O26</f>
+        <f>'Plan de charge'!O32</f>
         <v>0</v>
       </c>
       <c r="K5" s="8"/>
       <c r="L5" s="16"/>
       <c r="M5" s="7"/>
       <c r="N5" s="17" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="O5" s="18">
         <f>'Plan de charge'!G5</f>
@@ -10627,7 +10971,7 @@
       <c r="P5" s="4"/>
       <c r="V5" s="12"/>
       <c r="W5" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="X5" s="19">
         <f>+AC5-E5</f>
@@ -10636,7 +10980,7 @@
       <c r="Y5" s="13"/>
       <c r="AA5" s="12"/>
       <c r="AB5" s="20" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="AC5" s="21">
         <v>1500</v>
@@ -10646,7 +10990,7 @@
     <row r="6" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C6" s="7"/>
       <c r="D6" s="14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E6" s="15">
         <f>'Plan de charge'!O8</f>
@@ -10655,16 +10999,16 @@
       <c r="F6" s="8"/>
       <c r="H6" s="7"/>
       <c r="I6" s="22" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J6" s="23">
-        <f>'Plan de charge'!O28</f>
+        <f>'Plan de charge'!O34</f>
         <v>0</v>
       </c>
       <c r="K6" s="7"/>
       <c r="M6" s="7"/>
       <c r="N6" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="O6" s="24">
         <f>'Plan de charge'!G6</f>
@@ -10672,7 +11016,7 @@
       </c>
       <c r="P6" s="4"/>
       <c r="W6" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X6" s="19">
         <f>AC6-E9</f>
@@ -10681,7 +11025,7 @@
       <c r="Y6" s="13"/>
       <c r="AA6" s="12"/>
       <c r="AB6" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="AC6" s="19">
         <v>0</v>
@@ -10691,7 +11035,7 @@
     <row r="7" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C7" s="7"/>
       <c r="D7" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" s="15">
         <f>'Plan de charge'!O9</f>
@@ -10706,7 +11050,7 @@
       <c r="L7" s="25"/>
       <c r="M7" s="7"/>
       <c r="N7" s="22" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="O7" s="26">
         <f>SUM('Plan de charge'!G7:G13)</f>
@@ -10714,7 +11058,7 @@
       </c>
       <c r="P7" s="4"/>
       <c r="W7" s="14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="X7" s="19">
         <f>AC7-E6</f>
@@ -10723,7 +11067,7 @@
       <c r="Y7" s="13"/>
       <c r="AA7" s="12"/>
       <c r="AB7" s="20" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AC7" s="21">
         <f>E32-AC5-AC6-AC8-AC9</f>
@@ -10734,7 +11078,7 @@
     <row r="8" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C8" s="7"/>
       <c r="D8" s="14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E8" s="15">
         <f>'Plan de charge'!O11</f>
@@ -10742,14 +11086,14 @@
       </c>
       <c r="F8" s="8"/>
       <c r="H8" s="7"/>
-      <c r="I8" s="185" t="s">
-        <v>90</v>
-      </c>
-      <c r="J8" s="183"/>
+      <c r="I8" s="187" t="s">
+        <v>88</v>
+      </c>
+      <c r="J8" s="177"/>
       <c r="K8" s="8"/>
       <c r="M8" s="7"/>
       <c r="N8" s="27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O8" s="28">
         <f>SUM(O5:O7)</f>
@@ -10757,7 +11101,7 @@
       </c>
       <c r="P8" s="7"/>
       <c r="W8" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="X8" s="30">
         <f>SUM(X5:X7)</f>
@@ -10766,7 +11110,7 @@
       <c r="Y8" s="13"/>
       <c r="AA8" s="12"/>
       <c r="AB8" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="AC8" s="19">
         <f t="shared" ref="AC8:AC9" si="0">E7</f>
@@ -10777,7 +11121,7 @@
     <row r="9" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C9" s="7"/>
       <c r="D9" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E9" s="15">
         <f>'Plan de charge'!O10</f>
@@ -10785,11 +11129,11 @@
       </c>
       <c r="F9" s="8"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="186" t="e">
+      <c r="I9" s="183" t="e">
         <f>J5+J6-#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="J9" s="183"/>
+      <c r="J9" s="177"/>
       <c r="K9" s="8"/>
       <c r="M9" s="7"/>
       <c r="N9" s="4"/>
@@ -10801,7 +11145,7 @@
       <c r="Y9" s="13"/>
       <c r="AA9" s="12"/>
       <c r="AB9" s="14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="AC9" s="19">
         <f t="shared" si="0"/>
@@ -10812,7 +11156,7 @@
     <row r="10" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C10" s="7"/>
       <c r="D10" s="27" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E10" s="28">
         <f>SUM(E5:E9)</f>
@@ -10825,18 +11169,18 @@
       <c r="K10" s="34"/>
       <c r="M10" s="7"/>
       <c r="N10" s="182" t="s">
-        <v>92</v>
-      </c>
-      <c r="O10" s="183"/>
+        <v>90</v>
+      </c>
+      <c r="O10" s="177"/>
       <c r="P10" s="7"/>
-      <c r="W10" s="187" t="s">
-        <v>93</v>
-      </c>
-      <c r="X10" s="188"/>
+      <c r="W10" s="179" t="s">
+        <v>91</v>
+      </c>
+      <c r="X10" s="180"/>
       <c r="Y10" s="13"/>
       <c r="AA10" s="12"/>
       <c r="AB10" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="AC10" s="30">
         <f>SUM(AC5:AC9)</f>
@@ -10859,7 +11203,7 @@
       </c>
       <c r="P11" s="7"/>
       <c r="W11" s="35" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="X11" s="36" t="e">
         <f>D35-X12</f>
@@ -10874,13 +11218,13 @@
     <row r="12" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C12" s="7"/>
       <c r="D12" s="182" t="s">
-        <v>95</v>
-      </c>
-      <c r="E12" s="183"/>
+        <v>93</v>
+      </c>
+      <c r="E12" s="177"/>
       <c r="F12" s="8"/>
       <c r="M12" s="7"/>
       <c r="N12" s="14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O12" s="15">
         <f>'Plan de charge'!J10</f>
@@ -10888,7 +11232,7 @@
       </c>
       <c r="P12" s="7"/>
       <c r="W12" s="37" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="X12" s="38" t="e">
         <f>#REF!</f>
@@ -10896,31 +11240,31 @@
       </c>
       <c r="Y12" s="13"/>
       <c r="AA12" s="12"/>
-      <c r="AB12" s="184" t="s">
-        <v>95</v>
-      </c>
-      <c r="AC12" s="183"/>
+      <c r="AB12" s="181" t="s">
+        <v>93</v>
+      </c>
+      <c r="AC12" s="177"/>
       <c r="AD12" s="13"/>
     </row>
     <row r="13" spans="3:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C13" s="7"/>
       <c r="D13" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E13" s="15">
         <f>'Plan de charge'!O12</f>
         <v>0</v>
       </c>
       <c r="F13" s="8"/>
-      <c r="H13" s="192" t="s">
-        <v>97</v>
-      </c>
-      <c r="I13" s="193"/>
-      <c r="J13" s="193"/>
-      <c r="K13" s="183"/>
+      <c r="H13" s="175" t="s">
+        <v>95</v>
+      </c>
+      <c r="I13" s="176"/>
+      <c r="J13" s="176"/>
+      <c r="K13" s="177"/>
       <c r="M13" s="7"/>
       <c r="N13" s="14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="O13" s="15">
         <f>SUM('Plan de charge'!J6:J9)</f>
@@ -10928,7 +11272,7 @@
       </c>
       <c r="P13" s="7"/>
       <c r="W13" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="X13" s="30" t="e">
         <f>SUM(X11:X12)</f>
@@ -10937,7 +11281,7 @@
       <c r="Y13" s="13"/>
       <c r="AA13" s="12"/>
       <c r="AB13" s="17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AC13" s="39">
         <f t="shared" ref="AC13:AC14" si="1">E13</f>
@@ -10948,23 +11292,23 @@
     <row r="14" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C14" s="7"/>
       <c r="D14" s="14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E14" s="15">
-        <f>'Plan de charge'!O17+'Plan de charge'!O19</f>
+        <f>'Plan de charge'!O20+'Plan de charge'!O23</f>
         <v>0</v>
       </c>
       <c r="F14" s="8"/>
-      <c r="H14" s="194" t="e">
+      <c r="H14" s="178" t="e">
         <f>I9+D28</f>
         <v>#REF!</v>
       </c>
-      <c r="I14" s="193"/>
-      <c r="J14" s="193"/>
-      <c r="K14" s="183"/>
+      <c r="I14" s="176"/>
+      <c r="J14" s="176"/>
+      <c r="K14" s="177"/>
       <c r="M14" s="7"/>
       <c r="N14" s="14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="O14" s="15">
         <f>'Plan de charge'!J18+'Plan de charge'!J19</f>
@@ -10976,7 +11320,7 @@
       <c r="Y14" s="13"/>
       <c r="AA14" s="12"/>
       <c r="AB14" s="14" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="AC14" s="19">
         <f t="shared" si="1"/>
@@ -10987,30 +11331,30 @@
     <row r="15" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C15" s="7"/>
       <c r="D15" s="14" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E15" s="15">
-        <f>'Plan de charge'!O18+'Plan de charge'!O20</f>
+        <f>'Plan de charge'!O21+'Plan de charge'!O24</f>
         <v>0</v>
       </c>
       <c r="F15" s="8"/>
       <c r="M15" s="7"/>
       <c r="N15" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="O15" s="15">
         <f>'Plan de charge'!J35</f>
         <v>0</v>
       </c>
       <c r="P15" s="7"/>
-      <c r="W15" s="187" t="s">
-        <v>103</v>
-      </c>
-      <c r="X15" s="188"/>
+      <c r="W15" s="179" t="s">
+        <v>101</v>
+      </c>
+      <c r="X15" s="180"/>
       <c r="Y15" s="13"/>
       <c r="AA15" s="12"/>
       <c r="AB15" s="20" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="AC15" s="21" t="e">
         <f>X11</f>
@@ -11021,16 +11365,16 @@
     <row r="16" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C16" s="7"/>
       <c r="D16" s="14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E16" s="15">
-        <f>'Plan de charge'!O14+'Plan de charge'!O13</f>
+        <f>'Plan de charge'!O16+'Plan de charge'!O15</f>
         <v>0</v>
       </c>
       <c r="F16" s="8"/>
       <c r="M16" s="7"/>
       <c r="N16" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O16" s="15">
         <f>'Plan de charge'!J23-SUM(O11:O14)</f>
@@ -11038,7 +11382,7 @@
       </c>
       <c r="P16" s="7"/>
       <c r="W16" s="35" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="X16" s="36">
         <v>300</v>
@@ -11046,7 +11390,7 @@
       <c r="Y16" s="13"/>
       <c r="AA16" s="12"/>
       <c r="AB16" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="AC16" s="30" t="e">
         <f>SUM(AC13:AC15)</f>
@@ -11057,16 +11401,16 @@
     <row r="17" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C17" s="7"/>
       <c r="D17" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E17" s="15">
-        <f>'Plan de charge'!O15</f>
+        <f>'Plan de charge'!O17</f>
         <v>0</v>
       </c>
       <c r="F17" s="8"/>
       <c r="M17" s="7"/>
       <c r="N17" s="27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O17" s="28">
         <f>SUM(O11:O16)</f>
@@ -11074,7 +11418,7 @@
       </c>
       <c r="P17" s="7"/>
       <c r="W17" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="X17" s="40">
         <f>O19-X16</f>
@@ -11089,7 +11433,7 @@
     <row r="18" spans="3:30" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C18" s="7"/>
       <c r="D18" s="27" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E18" s="28">
         <f>SUM(E13:E17)</f>
@@ -11101,7 +11445,7 @@
       <c r="O18" s="41"/>
       <c r="P18" s="8"/>
       <c r="W18" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="X18" s="30">
         <f>X17+X16</f>
@@ -11109,10 +11453,10 @@
       </c>
       <c r="Y18" s="13"/>
       <c r="AA18" s="12"/>
-      <c r="AB18" s="184" t="s">
-        <v>107</v>
-      </c>
-      <c r="AC18" s="183"/>
+      <c r="AB18" s="181" t="s">
+        <v>105</v>
+      </c>
+      <c r="AC18" s="177"/>
       <c r="AD18" s="13"/>
     </row>
     <row r="19" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -11122,7 +11466,7 @@
       <c r="F19" s="8"/>
       <c r="M19" s="7"/>
       <c r="N19" s="42" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="O19" s="43">
         <f>O8-O17</f>
@@ -11135,7 +11479,7 @@
       <c r="Y19" s="13"/>
       <c r="AA19" s="12"/>
       <c r="AB19" s="14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="AC19" s="19">
         <f>E16</f>
@@ -11146,9 +11490,9 @@
     <row r="20" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C20" s="7"/>
       <c r="D20" s="182" t="s">
-        <v>107</v>
-      </c>
-      <c r="E20" s="183"/>
+        <v>105</v>
+      </c>
+      <c r="E20" s="177"/>
       <c r="F20" s="8"/>
       <c r="M20" s="32"/>
       <c r="N20" s="33"/>
@@ -11166,7 +11510,7 @@
     <row r="21" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C21" s="7"/>
       <c r="D21" s="17" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E21" s="18" t="e">
         <f>'Plan de charge'!#REF!</f>
@@ -11179,7 +11523,7 @@
       <c r="Y21" s="13"/>
       <c r="AA21" s="12"/>
       <c r="AB21" s="14" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="AC21" s="19">
         <f>E15</f>
@@ -11190,7 +11534,7 @@
     <row r="22" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C22" s="7"/>
       <c r="D22" s="14" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E22" s="15" t="e">
         <f>'Plan de charge'!#REF!</f>
@@ -11209,10 +11553,10 @@
     <row r="23" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C23" s="7"/>
       <c r="D23" s="14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E23" s="15">
-        <f>'Plan de charge'!O16</f>
+        <f>'Plan de charge'!O19</f>
         <v>0</v>
       </c>
       <c r="F23" s="8"/>
@@ -11222,7 +11566,7 @@
       <c r="Y23" s="13"/>
       <c r="AA23" s="12"/>
       <c r="AB23" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="AC23" s="19">
         <f>E17</f>
@@ -11233,7 +11577,7 @@
     <row r="24" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C24" s="7"/>
       <c r="D24" s="22" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E24" s="23" t="e">
         <f>'Plan de charge'!#REF!</f>
@@ -11252,7 +11596,7 @@
     <row r="25" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C25" s="7"/>
       <c r="D25" s="27" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E25" s="28" t="e">
         <f>SUM(E21:E24)</f>
@@ -11265,7 +11609,7 @@
       <c r="Y25" s="13"/>
       <c r="AA25" s="12"/>
       <c r="AB25" s="14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="AC25" s="19">
         <f>E23</f>
@@ -11284,7 +11628,7 @@
       <c r="Y26" s="13"/>
       <c r="AA26" s="12"/>
       <c r="AB26" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="AC26" s="30">
         <f>SUM(AC19:AC25)</f>
@@ -11294,10 +11638,10 @@
     </row>
     <row r="27" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C27" s="7"/>
-      <c r="D27" s="191" t="s">
-        <v>111</v>
-      </c>
-      <c r="E27" s="183"/>
+      <c r="D27" s="186" t="s">
+        <v>109</v>
+      </c>
+      <c r="E27" s="177"/>
       <c r="F27" s="8"/>
       <c r="V27" s="44"/>
       <c r="W27" s="45"/>
@@ -11310,11 +11654,11 @@
     </row>
     <row r="28" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C28" s="7"/>
-      <c r="D28" s="186" t="e">
+      <c r="D28" s="183" t="e">
         <f>E18+E10+E25</f>
         <v>#REF!</v>
       </c>
-      <c r="E28" s="183"/>
+      <c r="E28" s="177"/>
       <c r="F28" s="8"/>
       <c r="AA28" s="44"/>
       <c r="AB28" s="45"/>
@@ -11335,16 +11679,16 @@
     </row>
     <row r="31" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C31" s="7"/>
-      <c r="D31" s="189" t="s">
-        <v>112</v>
-      </c>
-      <c r="E31" s="183"/>
+      <c r="D31" s="184" t="s">
+        <v>110</v>
+      </c>
+      <c r="E31" s="177"/>
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="3:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C32" s="7"/>
       <c r="D32" s="47" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E32" s="48">
         <v>30000</v>
@@ -11359,19 +11703,19 @@
     </row>
     <row r="34" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C34" s="7"/>
-      <c r="D34" s="190" t="s">
-        <v>113</v>
-      </c>
-      <c r="E34" s="183"/>
+      <c r="D34" s="185" t="s">
+        <v>111</v>
+      </c>
+      <c r="E34" s="177"/>
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C35" s="7"/>
-      <c r="D35" s="186">
+      <c r="D35" s="183">
         <f>E10-E32</f>
         <v>-30000</v>
       </c>
-      <c r="E35" s="183"/>
+      <c r="E35" s="177"/>
       <c r="F35" s="8"/>
     </row>
     <row r="36" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -11435,7 +11779,7 @@
       <c r="P40" s="53"/>
       <c r="Q40" s="54"/>
       <c r="W40" s="56" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="X40" s="39">
         <f>AC10</f>
@@ -11460,7 +11804,7 @@
       <c r="P41" s="53"/>
       <c r="Q41" s="54"/>
       <c r="W41" s="57" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="X41" s="19">
         <f>AC13</f>
@@ -11485,7 +11829,7 @@
       <c r="P42" s="53"/>
       <c r="Q42" s="54"/>
       <c r="W42" s="57" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="X42" s="19" t="e">
         <f t="shared" ref="X42:X44" si="2">AC15</f>
@@ -11510,7 +11854,7 @@
       <c r="P43" s="53"/>
       <c r="Q43" s="54"/>
       <c r="W43" s="57" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="X43" s="19" t="e">
         <f t="shared" si="2"/>
@@ -11535,7 +11879,7 @@
       <c r="P44" s="53"/>
       <c r="Q44" s="54"/>
       <c r="W44" s="57" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X44" s="19">
         <f t="shared" si="2"/>
@@ -11560,7 +11904,7 @@
       <c r="P45" s="53"/>
       <c r="Q45" s="54"/>
       <c r="W45" s="57" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="X45" s="19">
         <f>AC21</f>
@@ -11585,7 +11929,7 @@
       <c r="P46" s="53"/>
       <c r="Q46" s="54"/>
       <c r="W46" s="58" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="X46" s="40">
         <f>AC19</f>
@@ -12159,14 +12503,14 @@
     <row r="80" spans="2:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="81" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D81" s="63" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E81" s="64">
         <f>E10</f>
         <v>0</v>
       </c>
       <c r="N81" s="63" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="O81" s="64">
         <f>SUM('Plan de charge'!O5:O11)</f>
@@ -12175,39 +12519,39 @@
     </row>
     <row r="82" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D82" s="65" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E82" s="66">
         <f>E13</f>
         <v>0</v>
       </c>
       <c r="N82" s="65" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="O82" s="66" t="e">
-        <f>SUM('Plan de charge'!O12:O15,'Plan de charge'!O17:O21,'Plan de charge'!#REF!)</f>
+        <f>SUM('Plan de charge'!O12:O17,'Plan de charge'!O20:O25,'Plan de charge'!#REF!)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="83" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D83" s="65" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E83" s="66">
         <f>E14+E15</f>
         <v>0</v>
       </c>
       <c r="N83" s="67" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="O83" s="68" t="e">
-        <f>'Plan de charge'!O16+'Plan de charge'!#REF!+'Plan de charge'!#REF!+I9+'Plan de charge'!#REF!</f>
+        <f>'Plan de charge'!O19+'Plan de charge'!#REF!+'Plan de charge'!#REF!+I9+'Plan de charge'!#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="84" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D84" s="65" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E84" s="66">
         <f>E17</f>
@@ -12218,46 +12562,46 @@
     </row>
     <row r="85" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D85" s="65" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E85" s="66">
         <f>E16</f>
         <v>0</v>
       </c>
       <c r="N85" s="63" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="O85" s="64" t="e">
-        <f>SUM('Plan de charge'!O5:O12,'Plan de charge'!O17,'Plan de charge'!O19,'Plan de charge'!#REF!,'Plan de charge'!#REF!)</f>
+        <f>SUM('Plan de charge'!O5:O12,'Plan de charge'!O20,'Plan de charge'!O23,'Plan de charge'!#REF!,'Plan de charge'!#REF!)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="86" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D86" s="65" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E86" s="66" t="e">
         <f>E21+E22</f>
         <v>#REF!</v>
       </c>
       <c r="N86" s="65" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="O86" s="66" t="e">
-        <f>SUM('Plan de charge'!O13:O16,'Plan de charge'!O18,'Plan de charge'!O20,'Plan de charge'!#REF!,'Plan de charge'!#REF!)</f>
+        <f>SUM('Plan de charge'!O15:O19,'Plan de charge'!O21,'Plan de charge'!O24,'Plan de charge'!#REF!,'Plan de charge'!#REF!)</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="87" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D87" s="65" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E87" s="66">
         <f t="shared" ref="E87:E88" si="3">E23</f>
         <v>0</v>
       </c>
       <c r="N87" s="65" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="O87" s="66" t="e">
         <f>I9</f>
@@ -12266,14 +12610,14 @@
     </row>
     <row r="88" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D88" s="65" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E88" s="66" t="e">
         <f t="shared" si="3"/>
         <v>#REF!</v>
       </c>
       <c r="N88" s="67" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="O88" s="68" t="e">
         <f>'Plan de charge'!#REF!</f>
@@ -12282,7 +12626,7 @@
     </row>
     <row r="89" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D89" s="67" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E89" s="68" t="e">
         <f>I9</f>
@@ -13202,22 +13546,6 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="W15:X15"/>
-    <mergeCell ref="AB18:AC18"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="W10:X10"/>
-    <mergeCell ref="AB12:AC12"/>
     <mergeCell ref="C2:F2"/>
     <mergeCell ref="H2:K2"/>
     <mergeCell ref="M2:P2"/>
@@ -13228,6 +13556,22 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="V2:Y2"/>
     <mergeCell ref="W4:X4"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="W10:X10"/>
+    <mergeCell ref="AB12:AC12"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="W15:X15"/>
+    <mergeCell ref="AB18:AC18"/>
+    <mergeCell ref="D20:E20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -13249,27 +13593,27 @@
   <sheetData>
     <row r="4" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B4" s="71" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B6" s="71" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B7" s="71" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B8" s="71" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B9" s="71" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -14290,26 +14634,26 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B2" s="195" t="s">
-        <v>137</v>
-      </c>
-      <c r="C2" s="183"/>
-      <c r="E2" s="196" t="s">
-        <v>79</v>
-      </c>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="180"/>
-      <c r="J2" s="196" t="s">
-        <v>138</v>
-      </c>
-      <c r="K2" s="179"/>
-      <c r="L2" s="179"/>
-      <c r="M2" s="180"/>
+      <c r="B2" s="192" t="s">
+        <v>135</v>
+      </c>
+      <c r="C2" s="177"/>
+      <c r="E2" s="193" t="s">
+        <v>77</v>
+      </c>
+      <c r="F2" s="189"/>
+      <c r="G2" s="189"/>
+      <c r="H2" s="190"/>
+      <c r="J2" s="193" t="s">
+        <v>136</v>
+      </c>
+      <c r="K2" s="189"/>
+      <c r="L2" s="189"/>
+      <c r="M2" s="190"/>
     </row>
     <row r="3" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="72" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C3" s="73" t="e">
         <f>Patrimoine!D28</f>
@@ -14326,26 +14670,26 @@
     </row>
     <row r="4" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="74" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C4" s="75" t="e">
         <f>Patrimoine!I9</f>
         <v>#REF!</v>
       </c>
       <c r="E4" s="12"/>
-      <c r="F4" s="190" t="s">
-        <v>141</v>
-      </c>
-      <c r="G4" s="183"/>
+      <c r="F4" s="185" t="s">
+        <v>139</v>
+      </c>
+      <c r="G4" s="177"/>
       <c r="H4" s="13"/>
       <c r="J4" s="12"/>
-      <c r="K4" s="184" t="s">
-        <v>81</v>
-      </c>
-      <c r="L4" s="183"/>
+      <c r="K4" s="181" t="s">
+        <v>79</v>
+      </c>
+      <c r="L4" s="177"/>
       <c r="M4" s="13"/>
       <c r="P4" s="17" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="Q4" s="76" t="b">
         <f>L10=Epargne_Precaution</f>
@@ -14354,22 +14698,22 @@
     </row>
     <row r="5" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="74" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C5" s="75" t="e">
         <f>Patrimoine_Total</f>
         <v>#REF!</v>
       </c>
       <c r="E5" s="12"/>
-      <c r="F5" s="186">
+      <c r="F5" s="183">
         <f>Montant_Investir</f>
         <v>-30000</v>
       </c>
-      <c r="G5" s="183"/>
+      <c r="G5" s="177"/>
       <c r="H5" s="13"/>
       <c r="J5" s="12"/>
       <c r="K5" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L5" s="15">
         <v>1000</v>
@@ -14377,7 +14721,7 @@
       <c r="M5" s="13"/>
       <c r="N5" s="16"/>
       <c r="P5" s="14" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q5" s="77" t="b">
         <f>G24=Montant_Investir</f>
@@ -14386,7 +14730,7 @@
     </row>
     <row r="6" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="74" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C6" s="75">
         <f>Epargne_Precaution</f>
@@ -14398,7 +14742,7 @@
       <c r="H6" s="13"/>
       <c r="J6" s="12"/>
       <c r="K6" s="14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L6" s="15">
         <f>G9+Patrimoine!E8</f>
@@ -14406,7 +14750,7 @@
       </c>
       <c r="M6" s="13"/>
       <c r="P6" s="14" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="Q6" s="77" t="b">
         <f>G31=Budget_Théorique</f>
@@ -14415,21 +14759,21 @@
     </row>
     <row r="7" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="78" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C7" s="79">
         <f>Montant_Investir</f>
         <v>-30000</v>
       </c>
       <c r="E7" s="12"/>
-      <c r="F7" s="184" t="s">
-        <v>84</v>
-      </c>
-      <c r="G7" s="183"/>
+      <c r="F7" s="181" t="s">
+        <v>82</v>
+      </c>
+      <c r="G7" s="177"/>
       <c r="H7" s="13"/>
       <c r="J7" s="12"/>
       <c r="K7" s="14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L7" s="15">
         <f>G10+Patrimoine!E6</f>
@@ -14438,7 +14782,7 @@
       <c r="M7" s="13"/>
       <c r="N7" s="25"/>
       <c r="P7" s="22" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Q7" s="80" t="e">
         <f>K31+G23=Patrimoine_Total</f>
@@ -14447,7 +14791,7 @@
     </row>
     <row r="8" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="78" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C8" s="79">
         <f>Budget_Théorique</f>
@@ -14455,7 +14799,7 @@
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G8" s="15">
         <f>L5-CC_0</f>
@@ -14464,7 +14808,7 @@
       <c r="H8" s="13"/>
       <c r="J8" s="12"/>
       <c r="K8" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L8" s="15">
         <f>G11+Patrimoine!E7</f>
@@ -14474,14 +14818,14 @@
     </row>
     <row r="9" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="81" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C9" s="82" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E9" s="12"/>
       <c r="F9" s="14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G9" s="15">
         <f>IF(LJ_0&gt;Epargne_Precaution-'Solution Patrimoniale'!L5,(Epargne_Precaution-'Solution Patrimoniale'!L5)-LJ_0,0)</f>
@@ -14490,7 +14834,7 @@
       <c r="H9" s="13"/>
       <c r="J9" s="12"/>
       <c r="K9" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L9" s="15">
         <f>G12+Patrimoine!E9</f>
@@ -14501,7 +14845,7 @@
     <row r="10" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="E10" s="12"/>
       <c r="F10" s="14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G10" s="15">
         <f>IF(SUM($L$5:L6)&lt;Epargne_Precaution,Epargne_Precaution-SUM($L$5:L6)-LA_0,-LA_0)</f>
@@ -14510,7 +14854,7 @@
       <c r="H10" s="13"/>
       <c r="J10" s="12"/>
       <c r="K10" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="L10" s="83">
         <f>SUM(L5:L9)</f>
@@ -14521,7 +14865,7 @@
     <row r="11" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="E11" s="12"/>
       <c r="F11" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G11" s="15">
         <f>IF(SUM($L$5:L7)&lt;Epargne_Precaution,Epargne_Precaution-SUM($L$5:L7)-LDD_0,-LDD_0)</f>
@@ -14536,7 +14880,7 @@
     <row r="12" spans="2:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E12" s="12"/>
       <c r="F12" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G12" s="15">
         <f>IF(SUM($L$5:L8)&lt;Epargne_Precaution,Epargne_Precaution-SUM($L$5:L8)-CEL_0,-CEL_0)</f>
@@ -14544,16 +14888,16 @@
       </c>
       <c r="H12" s="13"/>
       <c r="J12" s="12"/>
-      <c r="K12" s="184" t="s">
-        <v>95</v>
-      </c>
-      <c r="L12" s="183"/>
+      <c r="K12" s="181" t="s">
+        <v>93</v>
+      </c>
+      <c r="L12" s="177"/>
       <c r="M12" s="13"/>
     </row>
     <row r="13" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="E13" s="12"/>
       <c r="F13" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G13" s="83">
         <f>SUM(G8:G12)</f>
@@ -14562,7 +14906,7 @@
       <c r="H13" s="13"/>
       <c r="J13" s="12"/>
       <c r="K13" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L13" s="15">
         <f>G16+PEL_0</f>
@@ -14577,7 +14921,7 @@
       <c r="H14" s="13"/>
       <c r="J14" s="12"/>
       <c r="K14" s="14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L14" s="15">
         <f>G17+Ass_Vie_Euros_0</f>
@@ -14587,14 +14931,14 @@
     </row>
     <row r="15" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="E15" s="12"/>
-      <c r="F15" s="184" t="s">
-        <v>152</v>
-      </c>
-      <c r="G15" s="183"/>
+      <c r="F15" s="181" t="s">
+        <v>150</v>
+      </c>
+      <c r="G15" s="177"/>
       <c r="H15" s="13"/>
       <c r="J15" s="12"/>
       <c r="K15" s="14" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="L15" s="15">
         <f>G18</f>
@@ -14605,7 +14949,7 @@
     <row r="16" spans="2:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="E16" s="12"/>
       <c r="F16" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G16" s="15">
         <v>0</v>
@@ -14613,7 +14957,7 @@
       <c r="H16" s="13"/>
       <c r="J16" s="12"/>
       <c r="K16" s="14" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="L16" s="15">
         <f>G19+Ass_Vie_UC_0</f>
@@ -14624,7 +14968,7 @@
     <row r="17" spans="5:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="E17" s="12"/>
       <c r="F17" s="14" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="G17" s="15">
         <v>20000</v>
@@ -14632,7 +14976,7 @@
       <c r="H17" s="13"/>
       <c r="J17" s="12"/>
       <c r="K17" s="14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="L17" s="15">
         <f>G20+PEA_0</f>
@@ -14643,7 +14987,7 @@
     <row r="18" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E18" s="12"/>
       <c r="F18" s="14" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G18" s="15">
         <v>0</v>
@@ -14651,7 +14995,7 @@
       <c r="H18" s="13"/>
       <c r="J18" s="12"/>
       <c r="K18" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="L18" s="15">
         <f>G21+PEE_0</f>
@@ -14662,7 +15006,7 @@
     <row r="19" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E19" s="12"/>
       <c r="F19" s="14" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="G19" s="15">
         <v>0</v>
@@ -14670,7 +15014,7 @@
       <c r="H19" s="13"/>
       <c r="J19" s="12"/>
       <c r="K19" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="L19" s="83">
         <f>SUM(L13:L18)</f>
@@ -14681,7 +15025,7 @@
     <row r="20" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E20" s="12"/>
       <c r="F20" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G20" s="15">
         <v>0</v>
@@ -14695,23 +15039,23 @@
     <row r="21" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E21" s="12"/>
       <c r="F21" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G21" s="15">
         <v>0</v>
       </c>
       <c r="H21" s="13"/>
       <c r="J21" s="12"/>
-      <c r="K21" s="184" t="s">
-        <v>107</v>
-      </c>
-      <c r="L21" s="183"/>
+      <c r="K21" s="181" t="s">
+        <v>105</v>
+      </c>
+      <c r="L21" s="177"/>
       <c r="M21" s="13"/>
     </row>
     <row r="22" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E22" s="12"/>
       <c r="F22" s="14" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G22" s="15">
         <v>0</v>
@@ -14719,7 +15063,7 @@
       <c r="H22" s="13"/>
       <c r="J22" s="12"/>
       <c r="K22" s="17" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="L22" s="18" t="e">
         <f>PERP_Euros_0</f>
@@ -14730,7 +15074,7 @@
     <row r="23" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E23" s="12"/>
       <c r="F23" s="14" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G23" s="15">
         <v>6000</v>
@@ -14738,7 +15082,7 @@
       <c r="H23" s="13"/>
       <c r="J23" s="12"/>
       <c r="K23" s="14" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="L23" s="15" t="e">
         <f>PERP_UC_0</f>
@@ -14749,7 +15093,7 @@
     <row r="24" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E24" s="12"/>
       <c r="F24" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G24" s="83">
         <f>SUM(G16:G23)</f>
@@ -14758,7 +15102,7 @@
       <c r="H24" s="13"/>
       <c r="J24" s="12"/>
       <c r="K24" s="14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L24" s="15">
         <f>PERCO_0</f>
@@ -14773,7 +15117,7 @@
       <c r="H25" s="13"/>
       <c r="J25" s="12"/>
       <c r="K25" s="14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="L25" s="15" t="e">
         <f>SCPI_0+G22</f>
@@ -14783,14 +15127,14 @@
     </row>
     <row r="26" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E26" s="12"/>
-      <c r="F26" s="187" t="s">
-        <v>103</v>
-      </c>
-      <c r="G26" s="188"/>
+      <c r="F26" s="179" t="s">
+        <v>101</v>
+      </c>
+      <c r="G26" s="180"/>
       <c r="H26" s="13"/>
       <c r="J26" s="12"/>
       <c r="K26" s="14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L26" s="15" t="e">
         <f>Valeur_RP-#REF!</f>
@@ -14801,7 +15145,7 @@
     <row r="27" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E27" s="12"/>
       <c r="F27" s="17" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G27" s="18">
         <v>300</v>
@@ -14809,7 +15153,7 @@
       <c r="H27" s="13"/>
       <c r="J27" s="12"/>
       <c r="K27" s="22" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="L27" s="23" t="e">
         <f>Valeur_IL-#REF!</f>
@@ -14820,7 +15164,7 @@
     <row r="28" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E28" s="12"/>
       <c r="F28" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G28" s="15">
         <v>50</v>
@@ -14828,7 +15172,7 @@
       <c r="H28" s="13"/>
       <c r="J28" s="12"/>
       <c r="K28" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="L28" s="83" t="e">
         <f>SUM(L22:L27)</f>
@@ -14839,7 +15183,7 @@
     <row r="29" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E29" s="12"/>
       <c r="F29" s="14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G29" s="15">
         <v>300</v>
@@ -14853,7 +15197,7 @@
     <row r="30" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E30" s="12"/>
       <c r="F30" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G30" s="23">
         <f>Budget_Théorique-SUM(G27:G29)</f>
@@ -14861,16 +15205,16 @@
       </c>
       <c r="H30" s="13"/>
       <c r="J30" s="12"/>
-      <c r="K30" s="197" t="s">
-        <v>97</v>
-      </c>
-      <c r="L30" s="183"/>
+      <c r="K30" s="194" t="s">
+        <v>95</v>
+      </c>
+      <c r="L30" s="177"/>
       <c r="M30" s="13"/>
     </row>
     <row r="31" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E31" s="12"/>
       <c r="F31" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G31" s="83">
         <f>SUM(G27:G30)</f>
@@ -14878,11 +15222,11 @@
       </c>
       <c r="H31" s="13"/>
       <c r="J31" s="12"/>
-      <c r="K31" s="186" t="e">
+      <c r="K31" s="183" t="e">
         <f>L28+L19+L10</f>
         <v>#REF!</v>
       </c>
-      <c r="L31" s="183"/>
+      <c r="L31" s="177"/>
       <c r="M31" s="13"/>
     </row>
     <row r="32" spans="5:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -15630,7 +15974,7 @@
     <row r="76" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="77" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K77" s="63" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="L77" s="64">
         <f>L10</f>
@@ -15639,14 +15983,14 @@
     </row>
     <row r="78" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B78" s="63" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C78" s="64">
         <f>L10</f>
         <v>30000</v>
       </c>
       <c r="K78" s="65" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L78" s="66">
         <f>L19</f>
@@ -15655,14 +15999,14 @@
     </row>
     <row r="79" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B79" s="65" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C79" s="66">
         <f>L13</f>
         <v>0</v>
       </c>
       <c r="K79" s="67" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L79" s="68" t="e">
         <f>L28</f>
@@ -15671,7 +16015,7 @@
     </row>
     <row r="80" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B80" s="65" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C80" s="66">
         <f>SUM(L14:L16)</f>
@@ -15682,14 +16026,14 @@
     </row>
     <row r="81" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B81" s="65" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C81" s="66">
         <f>L18</f>
         <v>0</v>
       </c>
       <c r="K81" s="63" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="L81" s="64" t="e">
         <f>L10+L13+L14+L22</f>
@@ -15698,14 +16042,14 @@
     </row>
     <row r="82" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B82" s="65" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C82" s="66">
         <f>L17</f>
         <v>0</v>
       </c>
       <c r="K82" s="65" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="L82" s="66" t="e">
         <f>SUM(L15:L18)+L23+L24</f>
@@ -15714,14 +16058,14 @@
     </row>
     <row r="83" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B83" s="65" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C83" s="66" t="e">
         <f>L22+L23</f>
         <v>#REF!</v>
       </c>
       <c r="K83" s="65" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L83" s="66" t="e">
         <f>L26+L27</f>
@@ -15730,14 +16074,14 @@
     </row>
     <row r="84" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B84" s="65" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C84" s="66">
         <f t="shared" ref="C84:C85" si="0">L24</f>
         <v>0</v>
       </c>
       <c r="K84" s="67" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="L84" s="68" t="e">
         <f>+L25</f>
@@ -15746,7 +16090,7 @@
     </row>
     <row r="85" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B85" s="65" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C85" s="66" t="e">
         <f t="shared" si="0"/>
@@ -15755,7 +16099,7 @@
     </row>
     <row r="86" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B86" s="67" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C86" s="68" t="e">
         <f>L26+L27</f>

</xml_diff>